<commit_message>
feat(grimperium_mini): introduce multi-conformer mode for enhanced conformer analysis
- Added a new isolated module `multi_conformer.py` to run MOPAC on the best N CREST conformers without re-running CREST.
- Implemented a new CLI subcommand `multi-conformer` with options for input file, maximum conformers, and output directory.
- Enhanced the interactive TUI menu to include a multi-conformer mode option.
- Developed 21 unit tests to ensure functionality and robustness of the new feature.
- Updated the README and CHANGELOG to reflect the new capabilities and metrics.

These changes aim to improve the analysis of molecular conformers and streamline the computational workflow.
</commit_message>
<xml_diff>
--- a/data/grimperium_mini_pipeline_tcc.xlsx
+++ b/data/grimperium_mini_pipeline_tcc.xlsx
@@ -430,2322 +430,2194 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="10" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="14" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="22" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="22" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="22" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="16" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="14" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="18" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="18" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="20" hidden="0" customWidth="1"/>
-    <x:col min="22" max="22" width="52" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="4" t="str">
-        <x:v>Moléculas do CBThermo/TCC</x:v>
-      </x:c>
-      <x:c r="B1" s="4"/>
-      <x:c r="C1" s="4"/>
-      <x:c r="D1" s="4"/>
-      <x:c r="E1" s="4"/>
-      <x:c r="F1" s="4"/>
-      <x:c r="G1" s="4"/>
-      <x:c r="H1" s="4"/>
-      <x:c r="I1" s="4"/>
-      <x:c r="J1" s="4"/>
-      <x:c r="K1" s="4"/>
-      <x:c r="L1" s="4"/>
-      <x:c r="M1" s="4"/>
-      <x:c r="N1" s="4"/>
-      <x:c r="O1" s="4"/>
-      <x:c r="P1" s="4"/>
-      <x:c r="Q1" s="4"/>
-      <x:c r="R1" s="4"/>
-      <x:c r="S1" s="4"/>
-      <x:c r="T1" s="4"/>
-      <x:c r="U1" s="4"/>
-      <x:c r="V1" s="4"/>
-      <x:c r="W1" s="4"/>
-      <x:c r="X1" s="4"/>
-      <x:c r="Y1" s="4"/>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="10" t="str">
-        <x:v>Valores de referência e contribuição de grupos preservados da planilha original.</x:v>
-      </x:c>
-      <x:c r="B2" s="10"/>
-      <x:c r="C2" s="10"/>
-      <x:c r="D2" s="10"/>
-      <x:c r="E2" s="10"/>
-      <x:c r="F2" s="10"/>
-      <x:c r="G2" s="10"/>
-      <x:c r="H2" s="10"/>
-      <x:c r="I2" s="10"/>
-      <x:c r="J2" s="10"/>
-      <x:c r="K2" s="10"/>
-      <x:c r="L2" s="10"/>
-      <x:c r="M2" s="10"/>
-      <x:c r="N2" s="10"/>
-      <x:c r="O2" s="10"/>
-      <x:c r="P2" s="10"/>
-      <x:c r="Q2" s="10"/>
-      <x:c r="R2" s="10"/>
-      <x:c r="S2" s="10"/>
-      <x:c r="T2" s="10"/>
-      <x:c r="U2" s="10"/>
-      <x:c r="V2" s="10"/>
-      <x:c r="W2" s="10"/>
-      <x:c r="X2" s="10"/>
-      <x:c r="Y2" s="10"/>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="18" t="str">
-        <x:v>mol_id</x:v>
-      </x:c>
-      <x:c r="B4" s="18" t="str">
-        <x:v>molecule</x:v>
-      </x:c>
-      <x:c r="C4" s="18" t="str">
-        <x:v>smiles</x:v>
-      </x:c>
-      <x:c r="D4" s="18" t="str">
-        <x:v>formula</x:v>
-      </x:c>
-      <x:c r="E4" s="18" t="str">
-        <x:v>group</x:v>
-      </x:c>
-      <x:c r="F4" s="18" t="str">
-        <x:v>n_atoms</x:v>
-      </x:c>
-      <x:c r="G4" s="18" t="str">
-        <x:v>source_exp</x:v>
-      </x:c>
-      <x:c r="H4" s="18" t="str">
-        <x:v>Hf_exp_kJmol</x:v>
-      </x:c>
-      <x:c r="I4" s="18" t="str">
-        <x:v>Hf_JR_kJmol</x:v>
-      </x:c>
-      <x:c r="J4" s="18" t="str">
-        <x:v>Hf_CG_kJmol</x:v>
-      </x:c>
-      <x:c r="K4" s="18" t="str">
-        <x:v>Hf_MG_kJmol</x:v>
-      </x:c>
-      <x:c r="L4" s="18" t="str">
-        <x:v>Hf_AM1_TCC_VEGA_MOPAC_kJmol</x:v>
-      </x:c>
-      <x:c r="M4" s="18" t="str">
-        <x:v>Hf_PM3_TCC_VEGA_MOPAC_kJmol</x:v>
-      </x:c>
-      <x:c r="N4" s="18" t="str">
-        <x:v>Hf_PM7_TCC_VEGA_MOPAC_kJmol</x:v>
-      </x:c>
-      <x:c r="O4" s="18" t="str">
-        <x:v>Hf_RM1_TCC_VEGA_MOPAC_kJmol</x:v>
-      </x:c>
-      <x:c r="P4" s="18" t="str">
-        <x:v>AD_PM7_TCC_kJmol</x:v>
-      </x:c>
-      <x:c r="Q4" s="18" t="str">
-        <x:v>grimperium_original_mol_id</x:v>
-      </x:c>
-      <x:c r="R4" s="18" t="str">
-        <x:v>grimperium_original_status</x:v>
-      </x:c>
-      <x:c r="S4" s="18" t="str">
-        <x:v>grimperium_original_H298_pm7_kcalmol</x:v>
-      </x:c>
-      <x:c r="T4" s="18" t="str">
-        <x:v>grimperium_original_H298_pm7_kJmol</x:v>
-      </x:c>
-      <x:c r="U4" s="18" t="str">
-        <x:v>grimperium_original_H298_predicted_kcalmol</x:v>
-      </x:c>
-      <x:c r="V4" s="18" t="str">
-        <x:v>observacao</x:v>
-      </x:c>
-      <x:c r="W4" s="24"/>
-      <x:c r="X4" s="24"/>
-      <x:c r="Y4" s="24"/>
-      <x:c r="Z4" s="24"/>
-      <x:c r="AA4" s="24"/>
-      <x:c r="AB4" s="24"/>
-      <x:c r="AC4" s="24"/>
-      <x:c r="AD4" s="24"/>
-      <x:c r="AE4" s="24"/>
-      <x:c r="AF4" s="24"/>
-      <x:c r="AG4" s="24"/>
-      <x:c r="AH4" s="24"/>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" t="str">
-        <x:v>cbt_001</x:v>
-      </x:c>
-      <x:c r="B5" t="str">
-        <x:v>Acetic acid</x:v>
-      </x:c>
-      <x:c r="C5" t="str">
-        <x:v>CC(=O)O</x:v>
-      </x:c>
-      <x:c r="D5" t="str">
-        <x:v> C2H4O2</x:v>
-      </x:c>
-      <x:c r="E5" t="str">
-        <x:v>Acids</x:v>
-      </x:c>
-      <x:c r="F5" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="G5" t="str">
-        <x:v>CRC</x:v>
-      </x:c>
-      <x:c r="H5" s="26" t="n">
-        <x:v>-432.2</x:v>
-      </x:c>
-      <x:c r="I5" s="26" t="n">
-        <x:v>-434.88</x:v>
-      </x:c>
-      <x:c r="J5" s="26" t="n">
-        <x:v>-431.35400000000004</x:v>
-      </x:c>
-      <x:c r="K5" s="26" t="n">
-        <x:v>-426.861</x:v>
-      </x:c>
-      <x:c r="L5" s="26" t="n">
-        <x:v>-431.19347</x:v>
-      </x:c>
-      <x:c r="M5" s="26" t="n">
-        <x:v>-426.94471</x:v>
-      </x:c>
-      <x:c r="N5" s="26" t="n">
-        <x:v>-427.79466</x:v>
-      </x:c>
-      <x:c r="O5" s="26" t="n">
-        <x:v>-424.18656</x:v>
-      </x:c>
-      <x:c r="P5" s="26" t="n">
-        <x:v>4.405339999999967</x:v>
-      </x:c>
-      <x:c r="Q5" s="26" t="str"/>
-      <x:c r="R5" s="26" t="str"/>
-      <x:c r="S5" s="26"/>
-      <x:c r="T5" s="26"/>
-      <x:c r="U5" s="26"/>
-      <x:c r="V5" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" t="str">
-        <x:v>cbt_002</x:v>
-      </x:c>
-      <x:c r="B6" t="str">
-        <x:v>Propanoic acid</x:v>
-      </x:c>
-      <x:c r="C6" t="str">
-        <x:v>CCC(=O)O</x:v>
-      </x:c>
-      <x:c r="D6" t="str">
-        <x:v>C3H6O2</x:v>
-      </x:c>
-      <x:c r="E6" t="str">
-        <x:v>Acids</x:v>
-      </x:c>
-      <x:c r="F6" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="G6" t="str">
-        <x:v>CRC</x:v>
-      </x:c>
-      <x:c r="H6" s="26" t="n">
-        <x:v>-455.7</x:v>
-      </x:c>
-      <x:c r="I6" s="26" t="n">
-        <x:v>-455.52000000000004</x:v>
-      </x:c>
-      <x:c r="J6" s="26" t="n">
-        <x:v>-452.117</x:v>
-      </x:c>
-      <x:c r="K6" s="26" t="n">
-        <x:v>-447.69</x:v>
-      </x:c>
-      <x:c r="L6" s="26" t="n">
-        <x:v>-456.69109</x:v>
-      </x:c>
-      <x:c r="M6" s="26" t="n">
-        <x:v>-445.3205</x:v>
-      </x:c>
-      <x:c r="N6" s="26" t="n">
-        <x:v>-446.53103</x:v>
-      </x:c>
-      <x:c r="O6" s="26" t="n">
-        <x:v>-443.89516</x:v>
-      </x:c>
-      <x:c r="P6" s="26" t="n">
-        <x:v>9.168970000000002</x:v>
-      </x:c>
-      <x:c r="Q6" s="26" t="str">
-        <x:v>mol_01087</x:v>
-      </x:c>
-      <x:c r="R6" s="26" t="str">
-        <x:v>OK</x:v>
-      </x:c>
-      <x:c r="S6" s="26" t="n">
-        <x:v>-106.72</x:v>
-      </x:c>
-      <x:c r="T6" s="26" t="n">
-        <x:v>-446.51648</x:v>
-      </x:c>
-      <x:c r="U6" s="26" t="n">
-        <x:v>-106.750645</x:v>
-      </x:c>
-      <x:c r="V6" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="str">
-        <x:v>cbt_003</x:v>
-      </x:c>
-      <x:c r="B7" t="str">
-        <x:v>Butyric acid</x:v>
-      </x:c>
-      <x:c r="C7" t="str">
-        <x:v>CCCC(=O)O</x:v>
-      </x:c>
-      <x:c r="D7" t="str">
-        <x:v>C4H8O2</x:v>
-      </x:c>
-      <x:c r="E7" t="str">
-        <x:v>Acids</x:v>
-      </x:c>
-      <x:c r="F7" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="G7" t="str">
-        <x:v>PERRY</x:v>
-      </x:c>
-      <x:c r="H7" s="26" t="n">
-        <x:v>-475.8</x:v>
-      </x:c>
-      <x:c r="I7" s="26" t="n">
-        <x:v>-476.16</x:v>
-      </x:c>
-      <x:c r="J7" s="26" t="n">
-        <x:v>-472.88000000000005</x:v>
-      </x:c>
-      <x:c r="K7" s="26" t="n">
-        <x:v>-468.519</x:v>
-      </x:c>
-      <x:c r="L7" s="26" t="n">
-        <x:v>-485.54653</x:v>
-      </x:c>
-      <x:c r="M7" s="26" t="n">
-        <x:v>-467.96146</x:v>
-      </x:c>
-      <x:c r="N7" s="26" t="n">
-        <x:v>-468.50627</x:v>
-      </x:c>
-      <x:c r="O7" s="26" t="n">
-        <x:v>-464.59833</x:v>
-      </x:c>
-      <x:c r="P7" s="26" t="n">
-        <x:v>7.293730000000039</x:v>
-      </x:c>
-      <x:c r="Q7" s="26" t="str">
-        <x:v>mol_01110</x:v>
-      </x:c>
-      <x:c r="R7" s="26" t="str">
-        <x:v>OK</x:v>
-      </x:c>
-      <x:c r="S7" s="26" t="n">
-        <x:v>-111.98</x:v>
-      </x:c>
-      <x:c r="T7" s="26" t="n">
-        <x:v>-468.52432000000005</x:v>
-      </x:c>
-      <x:c r="U7" s="26" t="n">
-        <x:v>-111.161337</x:v>
-      </x:c>
-      <x:c r="V7" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="str">
-        <x:v>cbt_004</x:v>
-      </x:c>
-      <x:c r="B8" t="str">
-        <x:v>Pentanoic acid</x:v>
-      </x:c>
-      <x:c r="C8" t="str">
-        <x:v>CCCCC(=O)O</x:v>
-      </x:c>
-      <x:c r="D8" t="str">
-        <x:v>C5H10O2</x:v>
-      </x:c>
-      <x:c r="E8" t="str">
-        <x:v>Acids</x:v>
-      </x:c>
-      <x:c r="F8" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G8" t="str">
-        <x:v>PERRY</x:v>
-      </x:c>
-      <x:c r="H8" s="26" t="n">
-        <x:v>-491.3</x:v>
-      </x:c>
-      <x:c r="I8" s="26" t="n">
-        <x:v>-496.8</x:v>
-      </x:c>
-      <x:c r="J8" s="26" t="n">
-        <x:v>-493.64300000000003</x:v>
-      </x:c>
-      <x:c r="K8" s="26" t="n">
-        <x:v>-489.348</x:v>
-      </x:c>
-      <x:c r="L8" s="26" t="n">
-        <x:v>-514.08942</x:v>
-      </x:c>
-      <x:c r="M8" s="26" t="n">
-        <x:v>-490.54819</x:v>
-      </x:c>
-      <x:c r="N8" s="26" t="n">
-        <x:v>-489.3534</x:v>
-      </x:c>
-      <x:c r="O8" s="26" t="n">
-        <x:v>-487.6902</x:v>
-      </x:c>
-      <x:c r="P8" s="26" t="n">
-        <x:v>1.9465999999999894</x:v>
-      </x:c>
-      <x:c r="Q8" s="26" t="str">
-        <x:v>mol_01151</x:v>
-      </x:c>
-      <x:c r="R8" s="26" t="str">
-        <x:v>OK</x:v>
-      </x:c>
-      <x:c r="S8" s="26" t="n">
-        <x:v>-116.96</x:v>
-      </x:c>
-      <x:c r="T8" s="26" t="n">
-        <x:v>-489.36064</x:v>
-      </x:c>
-      <x:c r="U8" s="26" t="n">
-        <x:v>-115.302902</x:v>
-      </x:c>
-      <x:c r="V8" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="str">
-        <x:v>cbt_005</x:v>
-      </x:c>
-      <x:c r="B9" t="str">
-        <x:v>Hexanoic acid</x:v>
-      </x:c>
-      <x:c r="C9" t="str">
-        <x:v>CCCCCC(=O)O</x:v>
-      </x:c>
-      <x:c r="D9" t="str">
-        <x:v>C6H12O2</x:v>
-      </x:c>
-      <x:c r="E9" t="str">
-        <x:v>Acids</x:v>
-      </x:c>
-      <x:c r="F9" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="G9" t="str">
-        <x:v>PERRY</x:v>
-      </x:c>
-      <x:c r="H9" s="26" t="n">
-        <x:v>-511.9</x:v>
-      </x:c>
-      <x:c r="I9" s="26" t="n">
-        <x:v>-517.44</x:v>
-      </x:c>
-      <x:c r="J9" s="26" t="n">
-        <x:v>-514.406</x:v>
-      </x:c>
-      <x:c r="K9" s="26" t="n">
-        <x:v>-510.177</x:v>
-      </x:c>
-      <x:c r="L9" s="26" t="n">
-        <x:v>-542.79065</x:v>
-      </x:c>
-      <x:c r="M9" s="26" t="n">
-        <x:v>-513.24139</x:v>
-      </x:c>
-      <x:c r="N9" s="26" t="n">
-        <x:v>-510.9457</x:v>
-      </x:c>
-      <x:c r="O9" s="26" t="n">
-        <x:v>-508.62109</x:v>
-      </x:c>
-      <x:c r="P9" s="26" t="n">
-        <x:v>0.9542999999999893</x:v>
-      </x:c>
-      <x:c r="Q9" s="26" t="str">
-        <x:v>mol_01511</x:v>
-      </x:c>
-      <x:c r="R9" s="26" t="str">
-        <x:v>OK</x:v>
-      </x:c>
-      <x:c r="S9" s="26" t="n">
-        <x:v>-122.12</x:v>
-      </x:c>
-      <x:c r="T9" s="26" t="n">
-        <x:v>-510.95008</x:v>
-      </x:c>
-      <x:c r="U9" s="26"/>
-      <x:c r="V9" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str">
-        <x:v>cbt_006</x:v>
-      </x:c>
-      <x:c r="B10" t="str">
-        <x:v>Heptanoic acid</x:v>
-      </x:c>
-      <x:c r="C10" t="str">
-        <x:v>CCCCCCC(=O)O</x:v>
-      </x:c>
-      <x:c r="D10" t="str">
-        <x:v>C7H14O2</x:v>
-      </x:c>
-      <x:c r="E10" t="str">
-        <x:v>Acids</x:v>
-      </x:c>
-      <x:c r="F10" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="G10" t="str">
-        <x:v>PERRY</x:v>
-      </x:c>
-      <x:c r="H10" s="26" t="n">
-        <x:v>-536.2</x:v>
-      </x:c>
-      <x:c r="I10" s="26" t="n">
-        <x:v>-538.08</x:v>
-      </x:c>
-      <x:c r="J10" s="26" t="n">
-        <x:v>-535.169</x:v>
-      </x:c>
-      <x:c r="K10" s="26" t="n">
-        <x:v>-531.0060000000001</x:v>
-      </x:c>
-      <x:c r="L10" s="26" t="n">
-        <x:v>-571.46466</x:v>
-      </x:c>
-      <x:c r="M10" s="26" t="n">
-        <x:v>-535.93561</x:v>
-      </x:c>
-      <x:c r="N10" s="26" t="n">
-        <x:v>-532.2823</x:v>
-      </x:c>
-      <x:c r="O10" s="26" t="n">
-        <x:v>-529.4829</x:v>
-      </x:c>
-      <x:c r="P10" s="26" t="n">
-        <x:v>3.9177000000000817</x:v>
-      </x:c>
-      <x:c r="Q10" s="26" t="str">
-        <x:v>mol_01999</x:v>
-      </x:c>
-      <x:c r="R10" s="26" t="str">
-        <x:v>OK</x:v>
-      </x:c>
-      <x:c r="S10" s="26" t="n">
-        <x:v>-127.22</x:v>
-      </x:c>
-      <x:c r="T10" s="26" t="n">
-        <x:v>-532.28848</x:v>
-      </x:c>
-      <x:c r="U10" s="26"/>
-      <x:c r="V10" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" t="str">
-        <x:v>cbt_007</x:v>
-      </x:c>
-      <x:c r="B11" t="str">
-        <x:v>Octanoic acid</x:v>
-      </x:c>
-      <x:c r="C11" t="str">
-        <x:v>CCCCCCCC(=O)O</x:v>
-      </x:c>
-      <x:c r="D11" t="str">
-        <x:v>C8H16O2</x:v>
-      </x:c>
-      <x:c r="E11" t="str">
-        <x:v>Acids</x:v>
-      </x:c>
-      <x:c r="F11" t="n">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="G11" t="str">
-        <x:v>PERRY</x:v>
-      </x:c>
-      <x:c r="H11" s="26" t="n">
-        <x:v>-556</x:v>
-      </x:c>
-      <x:c r="I11" s="26" t="n">
-        <x:v>-558.72</x:v>
-      </x:c>
-      <x:c r="J11" s="26" t="n">
-        <x:v>-555.932</x:v>
-      </x:c>
-      <x:c r="K11" s="26" t="n">
-        <x:v>-551.835</x:v>
-      </x:c>
-      <x:c r="L11" s="26" t="n">
-        <x:v>-600.16472</x:v>
-      </x:c>
-      <x:c r="M11" s="26" t="n">
-        <x:v>-558.65708</x:v>
-      </x:c>
-      <x:c r="N11" s="26" t="n">
-        <x:v>-553.67659</x:v>
-      </x:c>
-      <x:c r="O11" s="26" t="n">
-        <x:v>-550.37463</x:v>
-      </x:c>
-      <x:c r="P11" s="26" t="n">
-        <x:v>2.323409999999967</x:v>
-      </x:c>
-      <x:c r="Q11" s="26" t="str">
-        <x:v>mol_02526</x:v>
-      </x:c>
-      <x:c r="R11" s="26" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="S11" s="26"/>
-      <x:c r="T11" s="26"/>
-      <x:c r="U11" s="26"/>
-      <x:c r="V11" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str">
-        <x:v>cbt_008</x:v>
-      </x:c>
-      <x:c r="B12" t="str">
-        <x:v>Dodecanoic acid</x:v>
-      </x:c>
-      <x:c r="C12" t="str">
-        <x:v>CCCCCCCCCCCC(=O)O</x:v>
-      </x:c>
-      <x:c r="D12" t="str">
-        <x:v>C12H24O2</x:v>
-      </x:c>
-      <x:c r="E12" t="str">
-        <x:v>Acids</x:v>
-      </x:c>
-      <x:c r="F12" t="n">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="G12" t="str">
-        <x:v>CRC</x:v>
-      </x:c>
-      <x:c r="H12" s="26" t="n">
-        <x:v>-642</x:v>
-      </x:c>
-      <x:c r="I12" s="26" t="n">
-        <x:v>-641.2800000000001</x:v>
-      </x:c>
-      <x:c r="J12" s="26" t="n">
-        <x:v>-638.984</x:v>
-      </x:c>
-      <x:c r="K12" s="26" t="n">
-        <x:v>-635.1510000000001</x:v>
-      </x:c>
-      <x:c r="L12" s="26" t="n">
-        <x:v>-711.97551</x:v>
-      </x:c>
-      <x:c r="M12" s="26" t="n">
-        <x:v>-647.41071</x:v>
-      </x:c>
-      <x:c r="N12" s="26" t="n">
-        <x:v>-636.75846</x:v>
-      </x:c>
-      <x:c r="O12" s="26" t="n">
-        <x:v>-630.763</x:v>
-      </x:c>
-      <x:c r="P12" s="26" t="n">
-        <x:v>5.241539999999986</x:v>
-      </x:c>
-      <x:c r="Q12" s="26" t="str">
-        <x:v>mol_19014</x:v>
-      </x:c>
-      <x:c r="R12" s="26" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="S12" s="26"/>
-      <x:c r="T12" s="26"/>
-      <x:c r="U12" s="26"/>
-      <x:c r="V12" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str">
-        <x:v>cbt_009</x:v>
-      </x:c>
-      <x:c r="B13" t="str">
-        <x:v>Tetradecanoic acid</x:v>
-      </x:c>
-      <x:c r="C13" t="str">
-        <x:v>CCCCCCCCCCCCCC(=O)O</x:v>
-      </x:c>
-      <x:c r="D13" t="str">
-        <x:v>C14H28O2</x:v>
-      </x:c>
-      <x:c r="E13" t="str">
-        <x:v>Acids</x:v>
-      </x:c>
-      <x:c r="F13" t="n">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="G13" t="str">
-        <x:v>CRC</x:v>
-      </x:c>
-      <x:c r="H13" s="26" t="n">
-        <x:v>-693.7</x:v>
-      </x:c>
-      <x:c r="I13" s="26" t="n">
-        <x:v>-682.5600000000001</x:v>
-      </x:c>
-      <x:c r="J13" s="26" t="n">
-        <x:v>-680.51</x:v>
-      </x:c>
-      <x:c r="K13" s="26" t="n">
-        <x:v>-676.809</x:v>
-      </x:c>
-      <x:c r="L13" s="26" t="n">
-        <x:v>-766.63135</x:v>
-      </x:c>
-      <x:c r="M13" s="26" t="n">
-        <x:v>-693.91212</x:v>
-      </x:c>
-      <x:c r="N13" s="26" t="n">
-        <x:v>-678.95566</x:v>
-      </x:c>
-      <x:c r="O13" s="26" t="n">
-        <x:v>-669.06647</x:v>
-      </x:c>
-      <x:c r="P13" s="26" t="n">
-        <x:v>14.74434000000008</x:v>
-      </x:c>
-      <x:c r="Q13" s="26" t="str"/>
-      <x:c r="R13" s="26" t="str"/>
-      <x:c r="S13" s="26"/>
-      <x:c r="T13" s="26"/>
-      <x:c r="U13" s="26"/>
-      <x:c r="V13" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="str">
-        <x:v>cbt_010</x:v>
-      </x:c>
-      <x:c r="B14" t="str">
-        <x:v>Hexadecanoic acid</x:v>
-      </x:c>
-      <x:c r="C14" t="str">
-        <x:v>CCCCCCCCCCCCCCCC(=O)O</x:v>
-      </x:c>
-      <x:c r="D14" t="str">
-        <x:v>C16H32O2</x:v>
-      </x:c>
-      <x:c r="E14" t="str">
-        <x:v>Acids</x:v>
-      </x:c>
-      <x:c r="F14" t="n">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="G14" t="str">
-        <x:v>CRC</x:v>
-      </x:c>
-      <x:c r="H14" s="26" t="n">
-        <x:v>-737.1</x:v>
-      </x:c>
-      <x:c r="I14" s="26" t="n">
-        <x:v>-723.8400000000001</x:v>
-      </x:c>
-      <x:c r="J14" s="26" t="n">
-        <x:v>-722.0360000000001</x:v>
-      </x:c>
-      <x:c r="K14" s="26" t="n">
-        <x:v>-718.467</x:v>
-      </x:c>
-      <x:c r="L14" s="26" t="n">
-        <x:v>-823.88158</x:v>
-      </x:c>
-      <x:c r="M14" s="26" t="n">
-        <x:v>-737.15746</x:v>
-      </x:c>
-      <x:c r="N14" s="26" t="n">
-        <x:v>-721.25162</x:v>
-      </x:c>
-      <x:c r="O14" s="26" t="n">
-        <x:v>-711.74763</x:v>
-      </x:c>
-      <x:c r="P14" s="26" t="n">
-        <x:v>15.84838000000002</x:v>
-      </x:c>
-      <x:c r="Q14" s="26" t="str">
-        <x:v>mol_19005</x:v>
-      </x:c>
-      <x:c r="R14" s="26" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="S14" s="26"/>
-      <x:c r="T14" s="26"/>
-      <x:c r="U14" s="26"/>
-      <x:c r="V14" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="str">
-        <x:v>cbt_011</x:v>
-      </x:c>
-      <x:c r="B15" t="str">
-        <x:v>Methanol</x:v>
-      </x:c>
-      <x:c r="C15" t="str">
-        <x:v>CO</x:v>
-      </x:c>
-      <x:c r="D15" t="str">
-        <x:v>CH4O</x:v>
-      </x:c>
-      <x:c r="E15" t="str">
-        <x:v>Alcohols</x:v>
-      </x:c>
-      <x:c r="F15" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="G15" t="str">
-        <x:v>PERRY</x:v>
-      </x:c>
-      <x:c r="H15" s="26" t="n">
-        <x:v>-200.94</x:v>
-      </x:c>
-      <x:c r="I15" s="26" t="n">
-        <x:v>-216.2</x:v>
-      </x:c>
-      <x:c r="J15" s="26" t="n">
-        <x:v>-216.534</x:v>
-      </x:c>
-      <x:c r="K15" s="26" t="n">
-        <x:v>-215.29</x:v>
-      </x:c>
-      <x:c r="L15" s="26" t="n">
-        <x:v>-238.71117</x:v>
-      </x:c>
-      <x:c r="M15" s="26" t="n">
-        <x:v>-217.14298</x:v>
-      </x:c>
-      <x:c r="N15" s="26" t="n">
-        <x:v>-204.75825</x:v>
-      </x:c>
-      <x:c r="O15" s="26" t="n">
-        <x:v>-209.73142</x:v>
-      </x:c>
-      <x:c r="P15" s="26" t="n">
-        <x:v>3.818250000000006</x:v>
-      </x:c>
-      <x:c r="Q15" s="26" t="str">
-        <x:v>mol_05665</x:v>
-      </x:c>
-      <x:c r="R15" s="26" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="S15" s="26"/>
-      <x:c r="T15" s="26"/>
-      <x:c r="U15" s="26"/>
-      <x:c r="V15" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" t="str">
-        <x:v>cbt_012</x:v>
-      </x:c>
-      <x:c r="B16" t="str">
-        <x:v>Ethanol</x:v>
-      </x:c>
-      <x:c r="C16" t="str">
-        <x:v>CCO</x:v>
-      </x:c>
-      <x:c r="D16" t="str">
-        <x:v>C2H6O</x:v>
-      </x:c>
-      <x:c r="E16" t="str">
-        <x:v>Alcohols</x:v>
-      </x:c>
-      <x:c r="F16" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="G16" t="str">
-        <x:v>PERRY</x:v>
-      </x:c>
-      <x:c r="H16" s="26" t="n">
-        <x:v>-234.95</x:v>
-      </x:c>
-      <x:c r="I16" s="26" t="n">
-        <x:v>-236.83999999999997</x:v>
-      </x:c>
-      <x:c r="J16" s="26" t="n">
-        <x:v>-237.297</x:v>
-      </x:c>
-      <x:c r="K16" s="26" t="n">
-        <x:v>-236.119</x:v>
-      </x:c>
-      <x:c r="L16" s="26" t="n">
-        <x:v>-268.83202</x:v>
-      </x:c>
-      <x:c r="M16" s="26" t="n">
-        <x:v>-245.83769</x:v>
-      </x:c>
-      <x:c r="N16" s="26" t="n">
-        <x:v>-242.07799</x:v>
-      </x:c>
-      <x:c r="O16" s="26" t="n">
-        <x:v>-241.44176</x:v>
-      </x:c>
-      <x:c r="P16" s="26" t="n">
-        <x:v>7.127990000000011</x:v>
-      </x:c>
-      <x:c r="Q16" s="26" t="str">
-        <x:v>mol_05309</x:v>
-      </x:c>
-      <x:c r="R16" s="26" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="S16" s="26"/>
-      <x:c r="T16" s="26"/>
-      <x:c r="U16" s="26"/>
-      <x:c r="V16" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" t="str">
-        <x:v>cbt_013</x:v>
-      </x:c>
-      <x:c r="B17" t="str">
-        <x:v>Glycerol</x:v>
-      </x:c>
-      <x:c r="C17" t="str">
-        <x:v>C(C(CO)O)O</x:v>
-      </x:c>
-      <x:c r="D17" t="str">
-        <x:v>C3H8O</x:v>
-      </x:c>
-      <x:c r="E17" t="str">
-        <x:v>Alcohols</x:v>
-      </x:c>
-      <x:c r="F17" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="G17" t="str">
-        <x:v>PERRY</x:v>
-      </x:c>
-      <x:c r="H17" s="26" t="n">
-        <x:v>-577.9</x:v>
-      </x:c>
-      <x:c r="I17" s="26" t="n">
-        <x:v>-567.22</x:v>
-      </x:c>
-      <x:c r="J17" s="26" t="n">
-        <x:v>-582.6099999999999</x:v>
-      </x:c>
-      <x:c r="K17" s="26" t="n">
-        <x:v>-582.7330000000001</x:v>
-      </x:c>
-      <x:c r="L17" s="26" t="n">
-        <x:v>-665.40715</x:v>
-      </x:c>
-      <x:c r="M17" s="26" t="n">
-        <x:v>-589.19924</x:v>
-      </x:c>
-      <x:c r="N17" s="26" t="n">
-        <x:v>-588.45026</x:v>
-      </x:c>
-      <x:c r="O17" s="26" t="n">
-        <x:v>-595.40912</x:v>
-      </x:c>
-      <x:c r="P17" s="26" t="n">
-        <x:v>10.55025999999998</x:v>
-      </x:c>
-      <x:c r="Q17" s="26" t="str"/>
-      <x:c r="R17" s="26" t="str"/>
-      <x:c r="S17" s="26"/>
-      <x:c r="T17" s="26"/>
-      <x:c r="U17" s="26"/>
-      <x:c r="V17" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" t="str">
-        <x:v>cbt_014</x:v>
-      </x:c>
-      <x:c r="B18" t="str">
-        <x:v>Propanol</x:v>
-      </x:c>
-      <x:c r="C18" t="str">
-        <x:v>CCCO</x:v>
-      </x:c>
-      <x:c r="D18" t="str">
-        <x:v>C3H8O</x:v>
-      </x:c>
-      <x:c r="E18" t="str">
-        <x:v>Alcohols</x:v>
-      </x:c>
-      <x:c r="F18" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="G18" t="str">
-        <x:v>PERRY</x:v>
-      </x:c>
-      <x:c r="H18" s="26" t="n">
-        <x:v>-254.6</x:v>
-      </x:c>
-      <x:c r="I18" s="26" t="n">
-        <x:v>-257.47999999999996</x:v>
-      </x:c>
-      <x:c r="J18" s="26" t="n">
-        <x:v>-258.06</x:v>
-      </x:c>
-      <x:c r="K18" s="26" t="n">
-        <x:v>-256.94800000000004</x:v>
-      </x:c>
-      <x:c r="L18" s="26" t="n">
-        <x:v>-297.83885</x:v>
-      </x:c>
-      <x:c r="M18" s="26" t="n">
-        <x:v>-268.20436</x:v>
-      </x:c>
-      <x:c r="N18" s="26" t="n">
-        <x:v>-262.4848</x:v>
-      </x:c>
-      <x:c r="O18" s="26" t="n">
-        <x:v>-262.4955</x:v>
-      </x:c>
-      <x:c r="P18" s="26" t="n">
-        <x:v>7.884800000000013</x:v>
-      </x:c>
-      <x:c r="Q18" s="26" t="str">
-        <x:v>mol_05320</x:v>
-      </x:c>
-      <x:c r="R18" s="26" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="S18" s="26"/>
-      <x:c r="T18" s="26"/>
-      <x:c r="U18" s="26"/>
-      <x:c r="V18" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" t="str">
-        <x:v>cbt_015</x:v>
-      </x:c>
-      <x:c r="B19" t="str">
-        <x:v>Butanol</x:v>
-      </x:c>
-      <x:c r="C19" t="str">
-        <x:v>CCCCO</x:v>
-      </x:c>
-      <x:c r="D19" t="str">
-        <x:v>C4H10O</x:v>
-      </x:c>
-      <x:c r="E19" t="str">
-        <x:v>Alcohols</x:v>
-      </x:c>
-      <x:c r="F19" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G19" t="str">
-        <x:v>PERRY</x:v>
-      </x:c>
-      <x:c r="H19" s="26" t="n">
-        <x:v>-275.1</x:v>
-      </x:c>
-      <x:c r="I19" s="26" t="n">
-        <x:v>-278.11999999999995</x:v>
-      </x:c>
-      <x:c r="J19" s="26" t="n">
-        <x:v>-278.82300000000004</x:v>
-      </x:c>
-      <x:c r="K19" s="26" t="n">
-        <x:v>-277.77700000000004</x:v>
-      </x:c>
-      <x:c r="L19" s="26" t="n">
-        <x:v>-326.4243</x:v>
-      </x:c>
-      <x:c r="M19" s="26" t="n">
-        <x:v>-290.86926</x:v>
-      </x:c>
-      <x:c r="N19" s="26" t="n">
-        <x:v>-283.15306</x:v>
-      </x:c>
-      <x:c r="O19" s="26" t="n">
-        <x:v>-283.30645</x:v>
-      </x:c>
-      <x:c r="P19" s="26" t="n">
-        <x:v>8.05305999999996</x:v>
-      </x:c>
-      <x:c r="Q19" s="26" t="str">
-        <x:v>mol_05337</x:v>
-      </x:c>
-      <x:c r="R19" s="26" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="S19" s="26"/>
-      <x:c r="T19" s="26"/>
-      <x:c r="U19" s="26"/>
-      <x:c r="V19" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" t="str">
-        <x:v>cbt_016</x:v>
-      </x:c>
-      <x:c r="B20" t="str">
-        <x:v>Pentanol</x:v>
-      </x:c>
-      <x:c r="C20" t="str">
-        <x:v>CCCCCO</x:v>
-      </x:c>
-      <x:c r="D20" t="str">
-        <x:v>C5H12O</x:v>
-      </x:c>
-      <x:c r="E20" t="str">
-        <x:v>Alcohols</x:v>
-      </x:c>
-      <x:c r="F20" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="G20" t="str">
-        <x:v>PERRY</x:v>
-      </x:c>
-      <x:c r="H20" s="26" t="n">
-        <x:v>-295.7</x:v>
-      </x:c>
-      <x:c r="I20" s="26" t="n">
-        <x:v>-298.75999999999993</x:v>
-      </x:c>
-      <x:c r="J20" s="26" t="n">
-        <x:v>-299.58600000000007</x:v>
-      </x:c>
-      <x:c r="K20" s="26" t="n">
-        <x:v>-298.60600000000005</x:v>
-      </x:c>
-      <x:c r="L20" s="26" t="n">
-        <x:v>-355.12297</x:v>
-      </x:c>
-      <x:c r="M20" s="26" t="n">
-        <x:v>-313.57749</x:v>
-      </x:c>
-      <x:c r="N20" s="26" t="n">
-        <x:v>-304.42055</x:v>
-      </x:c>
-      <x:c r="O20" s="26" t="n">
-        <x:v>-304.22328</x:v>
-      </x:c>
-      <x:c r="P20" s="26" t="n">
-        <x:v>8.720550000000003</x:v>
-      </x:c>
-      <x:c r="Q20" s="26" t="str">
-        <x:v>mol_05538</x:v>
-      </x:c>
-      <x:c r="R20" s="26" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="S20" s="26"/>
-      <x:c r="T20" s="26"/>
-      <x:c r="U20" s="26"/>
-      <x:c r="V20" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" t="str">
-        <x:v>cbt_017</x:v>
-      </x:c>
-      <x:c r="B21" t="str">
-        <x:v>Hexanol</x:v>
-      </x:c>
-      <x:c r="C21" t="str">
-        <x:v>CCCCCCO</x:v>
-      </x:c>
-      <x:c r="D21" t="str">
-        <x:v>C6H14O</x:v>
-      </x:c>
-      <x:c r="E21" t="str">
-        <x:v>Alcohols</x:v>
-      </x:c>
-      <x:c r="F21" t="n">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="G21" t="str">
-        <x:v>PERRY</x:v>
-      </x:c>
-      <x:c r="H21" s="26" t="n">
-        <x:v>-316.2</x:v>
-      </x:c>
-      <x:c r="I21" s="26" t="n">
-        <x:v>-319.4</x:v>
-      </x:c>
-      <x:c r="J21" s="26" t="n">
-        <x:v>-320.349</x:v>
-      </x:c>
-      <x:c r="K21" s="26" t="n">
-        <x:v>-319.43500000000006</x:v>
-      </x:c>
-      <x:c r="L21" s="26" t="n">
-        <x:v>-383.81376</x:v>
-      </x:c>
-      <x:c r="M21" s="26" t="n">
-        <x:v>-336.29314</x:v>
-      </x:c>
-      <x:c r="N21" s="26" t="n">
-        <x:v>-325.86172</x:v>
-      </x:c>
-      <x:c r="O21" s="26" t="n">
-        <x:v>-325.10002</x:v>
-      </x:c>
-      <x:c r="P21" s="26" t="n">
-        <x:v>9.661720000000003</x:v>
-      </x:c>
-      <x:c r="Q21" s="26" t="str">
-        <x:v>mol_05437</x:v>
-      </x:c>
-      <x:c r="R21" s="26" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="S21" s="26"/>
-      <x:c r="T21" s="26"/>
-      <x:c r="U21" s="26"/>
-      <x:c r="V21" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" t="str">
-        <x:v>cbt_018</x:v>
-      </x:c>
-      <x:c r="B22" t="str">
-        <x:v>Heptanol</x:v>
-      </x:c>
-      <x:c r="C22" t="str">
-        <x:v>CCCCCCCO</x:v>
-      </x:c>
-      <x:c r="D22" t="str">
-        <x:v>C7H16O</x:v>
-      </x:c>
-      <x:c r="E22" t="str">
-        <x:v>Alcohols</x:v>
-      </x:c>
-      <x:c r="F22" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="G22" t="str">
-        <x:v>PERRY</x:v>
-      </x:c>
-      <x:c r="H22" s="26" t="n">
-        <x:v>-336.8</x:v>
-      </x:c>
-      <x:c r="I22" s="26" t="n">
-        <x:v>-340.04</x:v>
-      </x:c>
-      <x:c r="J22" s="26" t="n">
-        <x:v>-341.112</x:v>
-      </x:c>
-      <x:c r="K22" s="26" t="n">
-        <x:v>-340.264</x:v>
-      </x:c>
-      <x:c r="L22" s="26" t="n">
-        <x:v>-412.51169</x:v>
-      </x:c>
-      <x:c r="M22" s="26" t="n">
-        <x:v>-359.01738</x:v>
-      </x:c>
-      <x:c r="N22" s="26" t="n">
-        <x:v>-347.16037</x:v>
-      </x:c>
-      <x:c r="O22" s="26" t="n">
-        <x:v>-345.98604</x:v>
-      </x:c>
-      <x:c r="P22" s="26" t="n">
-        <x:v>10.360369999999989</x:v>
-      </x:c>
-      <x:c r="Q22" s="26" t="str">
-        <x:v>mol_05573</x:v>
-      </x:c>
-      <x:c r="R22" s="26" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="S22" s="26"/>
-      <x:c r="T22" s="26"/>
-      <x:c r="U22" s="26"/>
-      <x:c r="V22" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" t="str">
-        <x:v>cbt_019</x:v>
-      </x:c>
-      <x:c r="B23" t="str">
-        <x:v>Octanol</x:v>
-      </x:c>
-      <x:c r="C23" t="str">
-        <x:v>CCCCCCCCO</x:v>
-      </x:c>
-      <x:c r="D23" t="str">
-        <x:v>C8H18O</x:v>
-      </x:c>
-      <x:c r="E23" t="str">
-        <x:v>Alcohols</x:v>
-      </x:c>
-      <x:c r="F23" t="n">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="G23" t="str">
-        <x:v>PERRY</x:v>
-      </x:c>
-      <x:c r="H23" s="26" t="n">
-        <x:v>-357.3</x:v>
-      </x:c>
-      <x:c r="I23" s="26" t="n">
-        <x:v>-360.68</x:v>
-      </x:c>
-      <x:c r="J23" s="26" t="n">
-        <x:v>-361.87500000000006</x:v>
-      </x:c>
-      <x:c r="K23" s="26" t="n">
-        <x:v>-361.093</x:v>
-      </x:c>
-      <x:c r="L23" s="26" t="n">
-        <x:v>-441.21152</x:v>
-      </x:c>
-      <x:c r="M23" s="26" t="n">
-        <x:v>-381.74613</x:v>
-      </x:c>
-      <x:c r="N23" s="26" t="n">
-        <x:v>-368.4913</x:v>
-      </x:c>
-      <x:c r="O23" s="26" t="n">
-        <x:v>-366.87266</x:v>
-      </x:c>
-      <x:c r="P23" s="26" t="n">
-        <x:v>11.191300000000012</x:v>
-      </x:c>
-      <x:c r="Q23" s="26" t="str"/>
-      <x:c r="R23" s="26" t="str"/>
-      <x:c r="S23" s="26"/>
-      <x:c r="T23" s="26"/>
-      <x:c r="U23" s="26"/>
-      <x:c r="V23" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" t="str">
-        <x:v>cbt_020</x:v>
-      </x:c>
-      <x:c r="B24" t="str">
-        <x:v>Methyl acetate</x:v>
-      </x:c>
-      <x:c r="C24" t="str">
-        <x:v>CC(=O)OC</x:v>
-      </x:c>
-      <x:c r="D24" t="str">
-        <x:v>C3H6O2</x:v>
-      </x:c>
-      <x:c r="E24" t="str">
-        <x:v>Esters</x:v>
-      </x:c>
-      <x:c r="F24" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="G24" t="str">
-        <x:v>PERRY</x:v>
-      </x:c>
-      <x:c r="H24" s="26" t="n">
-        <x:v>-411.9</x:v>
-      </x:c>
-      <x:c r="I24" s="26" t="n">
-        <x:v>-422.53000000000003</x:v>
-      </x:c>
-      <x:c r="J24" s="26" t="n">
-        <x:v>-424.84900000000005</x:v>
-      </x:c>
-      <x:c r="K24" s="26" t="n">
-        <x:v>-424.38800000000003</x:v>
-      </x:c>
-      <x:c r="L24" s="26" t="n">
-        <x:v>-403.84293</x:v>
-      </x:c>
-      <x:c r="M24" s="26" t="n">
-        <x:v>-393.95409</x:v>
-      </x:c>
-      <x:c r="N24" s="26" t="n">
-        <x:v>-405.05317</x:v>
-      </x:c>
-      <x:c r="O24" s="26" t="n">
-        <x:v>-394.69533</x:v>
-      </x:c>
-      <x:c r="P24" s="26" t="n">
-        <x:v>6.8468299999999545</x:v>
-      </x:c>
-      <x:c r="Q24" s="26" t="str"/>
-      <x:c r="R24" s="26" t="str"/>
-      <x:c r="S24" s="26"/>
-      <x:c r="T24" s="26"/>
-      <x:c r="U24" s="26"/>
-      <x:c r="V24" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" t="str">
-        <x:v>cbt_021</x:v>
-      </x:c>
-      <x:c r="B25" t="str">
-        <x:v>Methyl propionate</x:v>
-      </x:c>
-      <x:c r="C25" t="str">
-        <x:v>CCC(=O)OC</x:v>
-      </x:c>
-      <x:c r="D25" t="str">
-        <x:v>C4H8O2</x:v>
-      </x:c>
-      <x:c r="E25" t="str">
-        <x:v>Esters</x:v>
-      </x:c>
-      <x:c r="F25" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="G25" t="str">
-        <x:v>PERRY</x:v>
-      </x:c>
-      <x:c r="H25" s="26" t="n">
-        <x:v>-427.5</x:v>
-      </x:c>
-      <x:c r="I25" s="26" t="n">
-        <x:v>-443.17</x:v>
-      </x:c>
-      <x:c r="J25" s="26" t="n">
-        <x:v>-440.317</x:v>
-      </x:c>
-      <x:c r="K25" s="26" t="n">
-        <x:v>-443.61300000000006</x:v>
-      </x:c>
-      <x:c r="L25" s="26" t="n">
-        <x:v>-429.22249</x:v>
-      </x:c>
-      <x:c r="M25" s="26" t="n">
-        <x:v>-412.3485</x:v>
-      </x:c>
-      <x:c r="N25" s="26" t="n">
-        <x:v>-423.65167</x:v>
-      </x:c>
-      <x:c r="O25" s="26" t="n">
-        <x:v>-414.26053</x:v>
-      </x:c>
-      <x:c r="P25" s="26" t="n">
-        <x:v>3.848329999999976</x:v>
-      </x:c>
-      <x:c r="Q25" s="26" t="str">
-        <x:v>mol_03435</x:v>
-      </x:c>
-      <x:c r="R25" s="26" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="S25" s="26"/>
-      <x:c r="T25" s="26"/>
-      <x:c r="U25" s="26"/>
-      <x:c r="V25" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" t="str">
-        <x:v>cbt_022</x:v>
-      </x:c>
-      <x:c r="B26" t="str">
-        <x:v>Methyl butyrate</x:v>
-      </x:c>
-      <x:c r="C26" t="str">
-        <x:v>CCCC(=O)OC</x:v>
-      </x:c>
-      <x:c r="D26" t="str">
-        <x:v>C5H10O2</x:v>
-      </x:c>
-      <x:c r="E26" t="str">
-        <x:v>Esters</x:v>
-      </x:c>
-      <x:c r="F26" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G26" t="str">
-        <x:v>PERRY</x:v>
-      </x:c>
-      <x:c r="H26" s="26" t="n">
-        <x:v>-450.7</x:v>
-      </x:c>
-      <x:c r="I26" s="26" t="n">
-        <x:v>-463.81</x:v>
-      </x:c>
-      <x:c r="J26" s="26" t="n">
-        <x:v>-461.08</x:v>
-      </x:c>
-      <x:c r="K26" s="26" t="n">
-        <x:v>-464.442</x:v>
-      </x:c>
-      <x:c r="L26" s="26" t="n">
-        <x:v>-458.04864</x:v>
-      </x:c>
-      <x:c r="M26" s="26" t="n">
-        <x:v>-434.98867</x:v>
-      </x:c>
-      <x:c r="N26" s="26" t="n">
-        <x:v>-445.40576</x:v>
-      </x:c>
-      <x:c r="O26" s="26" t="n">
-        <x:v>-435.46894</x:v>
-      </x:c>
-      <x:c r="P26" s="26" t="n">
-        <x:v>5.294240000000002</x:v>
-      </x:c>
-      <x:c r="Q26" s="26" t="str">
-        <x:v>mol_03513</x:v>
-      </x:c>
-      <x:c r="R26" s="26" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="S26" s="26"/>
-      <x:c r="T26" s="26"/>
-      <x:c r="U26" s="26"/>
-      <x:c r="V26" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" t="str">
-        <x:v>cbt_023</x:v>
-      </x:c>
-      <x:c r="B27" t="str">
-        <x:v>Methyl pentanoate</x:v>
-      </x:c>
-      <x:c r="C27" t="str">
-        <x:v>CCCCC(=O)OC</x:v>
-      </x:c>
-      <x:c r="D27" t="str">
-        <x:v>C6H12O2</x:v>
-      </x:c>
-      <x:c r="E27" t="str">
-        <x:v>Esters</x:v>
-      </x:c>
-      <x:c r="F27" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="G27" t="str">
-        <x:v>CRC</x:v>
-      </x:c>
-      <x:c r="H27" s="26" t="n">
-        <x:v>-471.1</x:v>
-      </x:c>
-      <x:c r="I27" s="26" t="n">
-        <x:v>-484.45</x:v>
-      </x:c>
-      <x:c r="J27" s="26" t="n">
-        <x:v>-481.843</x:v>
-      </x:c>
-      <x:c r="K27" s="26" t="n">
-        <x:v>-485.271</x:v>
-      </x:c>
-      <x:c r="L27" s="26" t="n">
-        <x:v>-486.59503</x:v>
-      </x:c>
-      <x:c r="M27" s="26" t="n">
-        <x:v>-457.58244</x:v>
-      </x:c>
-      <x:c r="N27" s="26" t="n">
-        <x:v>-466.21327</x:v>
-      </x:c>
-      <x:c r="O27" s="26" t="n">
-        <x:v>-455.88914</x:v>
-      </x:c>
-      <x:c r="P27" s="26" t="n">
-        <x:v>4.88673</x:v>
-      </x:c>
-      <x:c r="Q27" s="26" t="str">
-        <x:v>mol_03606</x:v>
-      </x:c>
-      <x:c r="R27" s="26" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="S27" s="26"/>
-      <x:c r="T27" s="26"/>
-      <x:c r="U27" s="26"/>
-      <x:c r="V27" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" t="str">
-        <x:v>cbt_024</x:v>
-      </x:c>
-      <x:c r="B28" t="str">
-        <x:v>Methyl hexanoate</x:v>
-      </x:c>
-      <x:c r="C28" t="str">
-        <x:v>CCCCCC(=O)OC</x:v>
-      </x:c>
-      <x:c r="D28" t="str">
-        <x:v>C7H14O2</x:v>
-      </x:c>
-      <x:c r="E28" t="str">
-        <x:v>Esters</x:v>
-      </x:c>
-      <x:c r="F28" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="G28" t="str">
-        <x:v>CRC</x:v>
-      </x:c>
-      <x:c r="H28" s="26" t="n">
-        <x:v>-492.2</x:v>
-      </x:c>
-      <x:c r="I28" s="26" t="n">
-        <x:v>-505.09</x:v>
-      </x:c>
-      <x:c r="J28" s="26" t="n">
-        <x:v>-502.60600000000005</x:v>
-      </x:c>
-      <x:c r="K28" s="26" t="n">
-        <x:v>-506.1</x:v>
-      </x:c>
-      <x:c r="L28" s="26" t="n">
-        <x:v>-515.29703</x:v>
-      </x:c>
-      <x:c r="M28" s="26" t="n">
-        <x:v>-480.27905</x:v>
-      </x:c>
-      <x:c r="N28" s="26" t="n">
-        <x:v>-487.81117</x:v>
-      </x:c>
-      <x:c r="O28" s="26" t="n">
-        <x:v>-477.20211</x:v>
-      </x:c>
-      <x:c r="P28" s="26" t="n">
-        <x:v>4.3888299999999845</x:v>
-      </x:c>
-      <x:c r="Q28" s="26" t="str">
-        <x:v>mol_04136</x:v>
-      </x:c>
-      <x:c r="R28" s="26" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="S28" s="26"/>
-      <x:c r="T28" s="26"/>
-      <x:c r="U28" s="26"/>
-      <x:c r="V28" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" t="str">
-        <x:v>cbt_025</x:v>
-      </x:c>
-      <x:c r="B29" t="str">
-        <x:v>Methyl heptanoate</x:v>
-      </x:c>
-      <x:c r="C29" t="str">
-        <x:v>CCCCCCC(=O)OC</x:v>
-      </x:c>
-      <x:c r="D29" t="str">
-        <x:v>C8H16O2</x:v>
-      </x:c>
-      <x:c r="E29" t="str">
-        <x:v>Esters</x:v>
-      </x:c>
-      <x:c r="F29" t="n">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="G29" t="str">
-        <x:v>CRC</x:v>
-      </x:c>
-      <x:c r="H29" s="26" t="n">
-        <x:v>-515.5</x:v>
-      </x:c>
-      <x:c r="I29" s="26" t="n">
-        <x:v>-525.73</x:v>
-      </x:c>
-      <x:c r="J29" s="26" t="n">
-        <x:v>-523.3689999999999</x:v>
-      </x:c>
-      <x:c r="K29" s="26" t="n">
-        <x:v>-526.9290000000001</x:v>
-      </x:c>
-      <x:c r="L29" s="26" t="n">
-        <x:v>-543.97305</x:v>
-      </x:c>
-      <x:c r="M29" s="26" t="n">
-        <x:v>-502.97559</x:v>
-      </x:c>
-      <x:c r="N29" s="26" t="n">
-        <x:v>-509.13106</x:v>
-      </x:c>
-      <x:c r="O29" s="26" t="n">
-        <x:v>-498.07198</x:v>
-      </x:c>
-      <x:c r="P29" s="26" t="n">
-        <x:v>6.368940000000009</x:v>
-      </x:c>
-      <x:c r="Q29" s="26" t="str">
-        <x:v>mol_04742</x:v>
-      </x:c>
-      <x:c r="R29" s="26" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="S29" s="26"/>
-      <x:c r="T29" s="26"/>
-      <x:c r="U29" s="26"/>
-      <x:c r="V29" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" t="str">
-        <x:v>cbt_026</x:v>
-      </x:c>
-      <x:c r="B30" t="str">
-        <x:v>Methyl octanoate</x:v>
-      </x:c>
-      <x:c r="C30" t="str">
-        <x:v>CCCCCCCC(=O)OC</x:v>
-      </x:c>
-      <x:c r="D30" t="str">
-        <x:v>C9H18O2</x:v>
-      </x:c>
-      <x:c r="E30" t="str">
-        <x:v>Esters</x:v>
-      </x:c>
-      <x:c r="F30" t="n">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="G30" t="str">
-        <x:v>CRC</x:v>
-      </x:c>
-      <x:c r="H30" s="26" t="n">
-        <x:v>-533.9</x:v>
-      </x:c>
-      <x:c r="I30" s="26" t="n">
-        <x:v>-546.3700000000001</x:v>
-      </x:c>
-      <x:c r="J30" s="26" t="n">
-        <x:v>-544.132</x:v>
-      </x:c>
-      <x:c r="K30" s="26" t="n">
-        <x:v>-547.758</x:v>
-      </x:c>
-      <x:c r="L30" s="26" t="n">
-        <x:v>-572.67115</x:v>
-      </x:c>
-      <x:c r="M30" s="26" t="n">
-        <x:v>-525.69852</x:v>
-      </x:c>
-      <x:c r="N30" s="26" t="n">
-        <x:v>-530.5573</x:v>
-      </x:c>
-      <x:c r="O30" s="26" t="n">
-        <x:v>-518.94753</x:v>
-      </x:c>
-      <x:c r="P30" s="26" t="n">
-        <x:v>3.3426999999999225</x:v>
-      </x:c>
-      <x:c r="Q30" s="26" t="str"/>
-      <x:c r="R30" s="26" t="str"/>
-      <x:c r="S30" s="26"/>
-      <x:c r="T30" s="26"/>
-      <x:c r="U30" s="26"/>
-      <x:c r="V30" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" t="str">
-        <x:v>cbt_027</x:v>
-      </x:c>
-      <x:c r="B31" t="str">
-        <x:v>Methyl Dodecanoate</x:v>
-      </x:c>
-      <x:c r="C31" t="str">
-        <x:v>CCCCCCCCCCCC(=O)OC</x:v>
-      </x:c>
-      <x:c r="D31" t="str">
-        <x:v>C13H26O2</x:v>
-      </x:c>
-      <x:c r="E31" t="str">
-        <x:v>Esters</x:v>
-      </x:c>
-      <x:c r="F31" t="n">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="G31" t="str">
-        <x:v>CRC</x:v>
-      </x:c>
-      <x:c r="H31" s="26" t="n">
-        <x:v>-617.9</x:v>
-      </x:c>
-      <x:c r="I31" s="26" t="n">
-        <x:v>-628.9300000000001</x:v>
-      </x:c>
-      <x:c r="J31" s="26" t="n">
-        <x:v>-627.184</x:v>
-      </x:c>
-      <x:c r="K31" s="26" t="n">
-        <x:v>-631.0740000000001</x:v>
-      </x:c>
-      <x:c r="L31" s="26" t="n">
-        <x:v>-687.47505</x:v>
-      </x:c>
-      <x:c r="M31" s="26" t="n">
-        <x:v>-616.61431</x:v>
-      </x:c>
-      <x:c r="N31" s="26" t="n">
-        <x:v>-615.92062</x:v>
-      </x:c>
-      <x:c r="O31" s="26" t="n">
-        <x:v>-602.49831</x:v>
-      </x:c>
-      <x:c r="P31" s="26" t="n">
-        <x:v>1.979379999999992</x:v>
-      </x:c>
-      <x:c r="Q31" s="26" t="str">
-        <x:v>mol_19010</x:v>
-      </x:c>
-      <x:c r="R31" s="26" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="S31" s="26"/>
-      <x:c r="T31" s="26"/>
-      <x:c r="U31" s="26"/>
-      <x:c r="V31" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" t="str">
-        <x:v>cbt_028</x:v>
-      </x:c>
-      <x:c r="B32" t="str">
-        <x:v>Methyl Tetradecanoate</x:v>
-      </x:c>
-      <x:c r="C32" t="str">
-        <x:v>CCCCCCCCCCCCCC(=O)OC</x:v>
-      </x:c>
-      <x:c r="D32" t="str">
-        <x:v>C15H30O2</x:v>
-      </x:c>
-      <x:c r="E32" t="str">
-        <x:v>Esters</x:v>
-      </x:c>
-      <x:c r="F32" t="n">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="G32" t="str">
-        <x:v>CRC</x:v>
-      </x:c>
-      <x:c r="H32" s="26" t="n">
-        <x:v>-656.9</x:v>
-      </x:c>
-      <x:c r="I32" s="26" t="n">
-        <x:v>-670.21</x:v>
-      </x:c>
-      <x:c r="J32" s="26" t="n">
-        <x:v>-668.71</x:v>
-      </x:c>
-      <x:c r="K32" s="26" t="n">
-        <x:v>-672.732</x:v>
-      </x:c>
-      <x:c r="L32" s="26" t="n">
-        <x:v>-739.06414</x:v>
-      </x:c>
-      <x:c r="M32" s="26" t="n">
-        <x:v>-658.6227</x:v>
-      </x:c>
-      <x:c r="N32" s="26" t="n">
-        <x:v>-656.87245</x:v>
-      </x:c>
-      <x:c r="O32" s="26" t="n">
-        <x:v>-640.24608</x:v>
-      </x:c>
-      <x:c r="P32" s="26" t="n">
-        <x:v>0.02755000000001928</x:v>
-      </x:c>
-      <x:c r="Q32" s="26" t="str"/>
-      <x:c r="R32" s="26" t="str"/>
-      <x:c r="S32" s="26"/>
-      <x:c r="T32" s="26"/>
-      <x:c r="U32" s="26"/>
-      <x:c r="V32" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" t="str">
-        <x:v>cbt_029</x:v>
-      </x:c>
-      <x:c r="B33" t="str">
-        <x:v>Methyl Hexadecanoate</x:v>
-      </x:c>
-      <x:c r="C33" t="str">
-        <x:v>CCCCCCCCCCCCCCCC(=O)OC</x:v>
-      </x:c>
-      <x:c r="D33" t="str">
-        <x:v>C17H34O2</x:v>
-      </x:c>
-      <x:c r="E33" t="str">
-        <x:v>Esters</x:v>
-      </x:c>
-      <x:c r="F33" t="n">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="G33" t="str">
-        <x:v>NIST</x:v>
-      </x:c>
-      <x:c r="H33" s="26" t="n">
-        <x:v>-665.6</x:v>
-      </x:c>
-      <x:c r="I33" s="26" t="n">
-        <x:v>-711.49</x:v>
-      </x:c>
-      <x:c r="J33" s="26" t="n">
-        <x:v>-710.236</x:v>
-      </x:c>
-      <x:c r="K33" s="26" t="n">
-        <x:v>-714.3900000000001</x:v>
-      </x:c>
-      <x:c r="L33" s="26" t="n">
-        <x:v>-796.26075</x:v>
-      </x:c>
-      <x:c r="M33" s="26" t="n">
-        <x:v>-706.07494</x:v>
-      </x:c>
-      <x:c r="N33" s="26" t="n">
-        <x:v>-698.10851</x:v>
-      </x:c>
-      <x:c r="O33" s="26" t="n">
-        <x:v>-679.09472</x:v>
-      </x:c>
-      <x:c r="P33" s="26" t="n">
-        <x:v>32.50851</x:v>
-      </x:c>
-      <x:c r="Q33" s="26" t="str"/>
-      <x:c r="R33" s="26" t="str"/>
-      <x:c r="S33" s="26"/>
-      <x:c r="T33" s="26"/>
-      <x:c r="U33" s="26"/>
-      <x:c r="V33" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" t="str">
-        <x:v>cbt_030</x:v>
-      </x:c>
-      <x:c r="B34" t="str">
-        <x:v>Triacetin</x:v>
-      </x:c>
-      <x:c r="C34" t="str">
-        <x:v>CC(=O)OCC(COC(C)=O)OC(C)=O</x:v>
-      </x:c>
-      <x:c r="D34" t="str">
-        <x:v>C9H14O6</x:v>
-      </x:c>
-      <x:c r="E34" t="str">
-        <x:v>Triglycerides</x:v>
-      </x:c>
-      <x:c r="F34" t="n">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="G34" t="str">
-        <x:v>CRC</x:v>
-      </x:c>
-      <x:c r="H34" s="26" t="n">
-        <x:v>-1245</x:v>
-      </x:c>
-      <x:c r="I34" s="26" t="n">
-        <x:v>-1186.21</x:v>
-      </x:c>
-      <x:c r="J34" s="26" t="n">
-        <x:v>-1193.078</x:v>
-      </x:c>
-      <x:c r="K34" s="26" t="n">
-        <x:v>-1202.397</x:v>
-      </x:c>
-      <x:c r="L34" s="26" t="n">
-        <x:v>-1142.86094</x:v>
-      </x:c>
-      <x:c r="M34" s="26" t="n">
-        <x:v>-1100.06525</x:v>
-      </x:c>
-      <x:c r="N34" s="26" t="n">
-        <x:v>-1190.81269</x:v>
-      </x:c>
-      <x:c r="O34" s="26" t="n">
-        <x:v>-1130.8903</x:v>
-      </x:c>
-      <x:c r="P34" s="26" t="n">
-        <x:v>54.187310000000025</x:v>
-      </x:c>
-      <x:c r="Q34" s="26" t="str">
-        <x:v>mol_19015</x:v>
-      </x:c>
-      <x:c r="R34" s="26" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="S34" s="26"/>
-      <x:c r="T34" s="26"/>
-      <x:c r="U34" s="26"/>
-      <x:c r="V34" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" t="str">
-        <x:v>cbt_031</x:v>
-      </x:c>
-      <x:c r="B35" t="str">
-        <x:v>Tributyrin</x:v>
-      </x:c>
-      <x:c r="C35" t="str">
-        <x:v>CCCC(=O)OCC(COC(=O)CCC)OC(=O)CCC</x:v>
-      </x:c>
-      <x:c r="D35" t="str">
-        <x:v>C15H26O6</x:v>
-      </x:c>
-      <x:c r="E35" t="str">
-        <x:v>Triglycerides</x:v>
-      </x:c>
-      <x:c r="F35" t="n">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="G35" t="str">
-        <x:v>NIST</x:v>
-      </x:c>
-      <x:c r="H35" s="26" t="n">
-        <x:v>-1388.9</x:v>
-      </x:c>
-      <x:c r="I35" s="26" t="n">
-        <x:v>-1310.0500000000002</x:v>
-      </x:c>
-      <x:c r="J35" s="26" t="n">
-        <x:v>-1312.3609999999999</x:v>
-      </x:c>
-      <x:c r="K35" s="26" t="n">
-        <x:v>-1325.767</x:v>
-      </x:c>
-      <x:c r="L35" s="26" t="n">
-        <x:v>-1299.98751</x:v>
-      </x:c>
-      <x:c r="M35" s="26" t="n">
-        <x:v>-1229.83066</x:v>
-      </x:c>
-      <x:c r="N35" s="26" t="n">
-        <x:v>-1303.39424</x:v>
-      </x:c>
-      <x:c r="O35" s="26" t="n">
-        <x:v>-1252.52058</x:v>
-      </x:c>
-      <x:c r="P35" s="26" t="n">
-        <x:v>85.50576000000001</x:v>
-      </x:c>
-      <x:c r="Q35" s="26" t="str"/>
-      <x:c r="R35" s="26" t="str"/>
-      <x:c r="S35" s="26"/>
-      <x:c r="T35" s="26"/>
-      <x:c r="U35" s="26"/>
-      <x:c r="V35" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" t="str">
-        <x:v>cbt_032</x:v>
-      </x:c>
-      <x:c r="B36" t="str">
-        <x:v>Trilaurin</x:v>
-      </x:c>
-      <x:c r="C36" t="str">
-        <x:v>CCCCCCCCCCCC(=O)OCC(COC(=O)CCCCCCCCCCC)OC(=O)CCCCCCCCCCC</x:v>
-      </x:c>
-      <x:c r="D36" t="str">
-        <x:v>C39H74O6</x:v>
-      </x:c>
-      <x:c r="E36" t="str">
-        <x:v>Triglycerides</x:v>
-      </x:c>
-      <x:c r="F36" t="n">
-        <x:v>119</x:v>
-      </x:c>
-      <x:c r="G36" t="str">
-        <x:v>NIST</x:v>
-      </x:c>
-      <x:c r="H36" s="26" t="n">
-        <x:v>-1887.4899999999998</x:v>
-      </x:c>
-      <x:c r="I36" s="26" t="n">
-        <x:v>-1805.41</x:v>
-      </x:c>
-      <x:c r="J36" s="26" t="n">
-        <x:v>-1810.6729999999998</x:v>
-      </x:c>
-      <x:c r="K36" s="26" t="n">
-        <x:v>-1825.663</x:v>
-      </x:c>
-      <x:c r="L36" s="26" t="n">
-        <x:v>-1990.7189</x:v>
-      </x:c>
-      <x:c r="M36" s="26" t="n">
-        <x:v>-1768.19792</x:v>
-      </x:c>
-      <x:c r="N36" s="26" t="n">
-        <x:v>-1824.35589</x:v>
-      </x:c>
-      <x:c r="O36" s="26" t="n">
-        <x:v>-1755.12124</x:v>
-      </x:c>
-      <x:c r="P36" s="26" t="n">
-        <x:v>63.13410999999974</x:v>
-      </x:c>
-      <x:c r="Q36" s="26" t="str"/>
-      <x:c r="R36" s="26" t="str"/>
-      <x:c r="S36" s="26"/>
-      <x:c r="T36" s="26"/>
-      <x:c r="U36" s="26"/>
-      <x:c r="V36" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" t="str">
-        <x:v>cbt_033</x:v>
-      </x:c>
-      <x:c r="B37" t="str">
-        <x:v>Trimyristin</x:v>
-      </x:c>
-      <x:c r="C37" t="str">
-        <x:v>CCCCCCCCCCCCCC(=O)OCC(COC(=O)CCCCCCCCCCCCC)OC(=O)CCCCCCCCCCCCC</x:v>
-      </x:c>
-      <x:c r="D37" t="str">
-        <x:v>C45H86O6</x:v>
-      </x:c>
-      <x:c r="E37" t="str">
-        <x:v>Triglycerides</x:v>
-      </x:c>
-      <x:c r="F37" t="n">
-        <x:v>137</x:v>
-      </x:c>
-      <x:c r="G37" t="str">
-        <x:v>NIST</x:v>
-      </x:c>
-      <x:c r="H37" s="26" t="n">
-        <x:v>-2003.6000000000001</x:v>
-      </x:c>
-      <x:c r="I37" s="26" t="n">
-        <x:v>-1929.25</x:v>
-      </x:c>
-      <x:c r="J37" s="26" t="n">
-        <x:v>-1935.2509999999997</x:v>
-      </x:c>
-      <x:c r="K37" s="26" t="n">
-        <x:v>-1950.6370000000002</x:v>
-      </x:c>
-      <x:c r="L37" s="26" t="n">
-        <x:v>-2162.9471</x:v>
-      </x:c>
-      <x:c r="M37" s="26" t="n">
-        <x:v>-1904.63415</x:v>
-      </x:c>
-      <x:c r="N37" s="26" t="n">
-        <x:v>-1955.36378</x:v>
-      </x:c>
-      <x:c r="O37" s="26" t="n">
-        <x:v>-1886.10792</x:v>
-      </x:c>
-      <x:c r="P37" s="26" t="n">
-        <x:v>48.23622000000023</x:v>
-      </x:c>
-      <x:c r="Q37" s="26" t="str"/>
-      <x:c r="R37" s="26" t="str"/>
-      <x:c r="S37" s="26"/>
-      <x:c r="T37" s="26"/>
-      <x:c r="U37" s="26"/>
-      <x:c r="V37" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38">
-      <x:c r="A38" t="str">
-        <x:v>cbt_034</x:v>
-      </x:c>
-      <x:c r="B38" t="str">
-        <x:v>Tripalmitin</x:v>
-      </x:c>
-      <x:c r="C38" t="str">
-        <x:v>CCCCCCCCCCCCCCCC(=O)OCC(COC(=O)CCCCCCCCCCCCCCC)OC(=O)CCCCCCCCCCCCCCC</x:v>
-      </x:c>
-      <x:c r="D38" t="str">
-        <x:v>C51H98O6</x:v>
-      </x:c>
-      <x:c r="E38" t="str">
-        <x:v>Triglycerides</x:v>
-      </x:c>
-      <x:c r="F38" t="n">
-        <x:v>155</x:v>
-      </x:c>
-      <x:c r="G38" t="str">
-        <x:v>NIST</x:v>
-      </x:c>
-      <x:c r="H38" s="26" t="n">
-        <x:v>-2089</x:v>
-      </x:c>
-      <x:c r="I38" s="26" t="n">
-        <x:v>-2053.09</x:v>
-      </x:c>
-      <x:c r="J38" s="26" t="n">
-        <x:v>-2059.8289999999997</x:v>
-      </x:c>
-      <x:c r="K38" s="26" t="n">
-        <x:v>-2075.611</x:v>
-      </x:c>
-      <x:c r="L38" s="26" t="n">
-        <x:v>-2335.22083</x:v>
-      </x:c>
-      <x:c r="M38" s="26" t="n">
-        <x:v>-2041.06221</x:v>
-      </x:c>
-      <x:c r="N38" s="26" t="n">
-        <x:v>-2082.95641</x:v>
-      </x:c>
-      <x:c r="O38" s="26" t="n">
-        <x:v>-2008.36722</x:v>
-      </x:c>
-      <x:c r="P38" s="26" t="n">
-        <x:v>6.043590000000222</x:v>
-      </x:c>
-      <x:c r="Q38" s="26" t="str"/>
-      <x:c r="R38" s="26" t="str"/>
-      <x:c r="S38" s="26"/>
-      <x:c r="T38" s="26"/>
-      <x:c r="U38" s="26"/>
-      <x:c r="V38" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" t="str">
-        <x:v>cbt_035</x:v>
-      </x:c>
-      <x:c r="B39" t="str">
-        <x:v>Water</x:v>
-      </x:c>
-      <x:c r="C39" t="str">
-        <x:v>O</x:v>
-      </x:c>
-      <x:c r="D39" t="str">
-        <x:v>H2O</x:v>
-      </x:c>
-      <x:c r="E39" t="str">
-        <x:v>Auxiliary</x:v>
-      </x:c>
-      <x:c r="F39" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G39" t="str">
-        <x:v>NIST</x:v>
-      </x:c>
-      <x:c r="H39" s="26" t="n">
-        <x:v>-241.83</x:v>
-      </x:c>
-      <x:c r="I39" s="26" t="n">
-        <x:v>-241.83</x:v>
-      </x:c>
-      <x:c r="J39" s="26" t="n">
-        <x:v>-241.83</x:v>
-      </x:c>
-      <x:c r="K39" s="26" t="n">
-        <x:v>-241.83</x:v>
-      </x:c>
-      <x:c r="L39" s="26" t="n">
-        <x:v>-241.83</x:v>
-      </x:c>
-      <x:c r="M39" s="26" t="n">
-        <x:v>-241.83</x:v>
-      </x:c>
-      <x:c r="N39" s="26" t="n">
-        <x:v>-241.83</x:v>
-      </x:c>
-      <x:c r="O39" s="26" t="n">
-        <x:v>-241.83</x:v>
-      </x:c>
-      <x:c r="P39" s="26" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Q39" s="26" t="str"/>
-      <x:c r="R39" s="26" t="str"/>
-      <x:c r="S39" s="26"/>
-      <x:c r="T39" s="26"/>
-      <x:c r="U39" s="26"/>
-      <x:c r="V39" t="str">
-        <x:v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:Y1"/>
-    <x:mergeCell ref="A2:Y2"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="42" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="10" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="15" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="14" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="22" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="22" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="22" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="22" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="16" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="18" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="14" hidden="0" customWidth="1"/>
+    <col min="19" max="19" width="18" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="18" hidden="0" customWidth="1"/>
+    <col min="21" max="21" width="20" hidden="0" customWidth="1"/>
+    <col min="22" max="22" width="52" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="str">
+        <v>Moléculas do CBThermo/TCC</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4"/>
+      <c r="R1" s="4"/>
+      <c r="S1" s="4"/>
+      <c r="T1" s="4"/>
+      <c r="U1" s="4"/>
+      <c r="V1" s="4"/>
+      <c r="W1" s="4"/>
+      <c r="X1" s="4"/>
+      <c r="Y1" s="4"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="str">
+        <v>Valores de referência e contribuição de grupos preservados da planilha original.</v>
+      </c>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="10"/>
+      <c r="P2" s="10"/>
+      <c r="Q2" s="10"/>
+      <c r="R2" s="10"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
+      <c r="V2" s="10"/>
+      <c r="W2" s="10"/>
+      <c r="X2" s="10"/>
+      <c r="Y2" s="10"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="18" t="str">
+        <v>mol_id</v>
+      </c>
+      <c r="B4" s="18" t="str">
+        <v>molecule</v>
+      </c>
+      <c r="C4" s="18" t="str">
+        <v>smiles</v>
+      </c>
+      <c r="D4" s="18" t="str">
+        <v>formula</v>
+      </c>
+      <c r="E4" s="18" t="str">
+        <v>group</v>
+      </c>
+      <c r="F4" s="18" t="str">
+        <v>n_atoms</v>
+      </c>
+      <c r="G4" s="18" t="str">
+        <v>source_exp</v>
+      </c>
+      <c r="H4" s="18" t="str">
+        <v>Hf_exp_kJmol</v>
+      </c>
+      <c r="I4" s="18" t="str">
+        <v>Hf_JR_kJmol</v>
+      </c>
+      <c r="J4" s="18" t="str">
+        <v>Hf_CG_kJmol</v>
+      </c>
+      <c r="K4" s="18" t="str">
+        <v>Hf_MG_kJmol</v>
+      </c>
+      <c r="L4" s="18" t="str">
+        <v>Hf_AM1_TCC_VEGA_MOPAC_kJmol</v>
+      </c>
+      <c r="M4" s="18" t="str">
+        <v>Hf_PM3_TCC_VEGA_MOPAC_kJmol</v>
+      </c>
+      <c r="N4" s="18" t="str">
+        <v>Hf_PM7_TCC_VEGA_MOPAC_kJmol</v>
+      </c>
+      <c r="O4" s="18" t="str">
+        <v>Hf_RM1_TCC_VEGA_MOPAC_kJmol</v>
+      </c>
+      <c r="P4" s="18" t="str">
+        <v>AD_PM7_TCC_kJmol</v>
+      </c>
+      <c r="Q4" s="18" t="str">
+        <v>grimperium_original_mol_id</v>
+      </c>
+      <c r="R4" s="18" t="str">
+        <v>grimperium_original_status</v>
+      </c>
+      <c r="S4" s="18" t="str">
+        <v>grimperium_original_H298_pm7_kcalmol</v>
+      </c>
+      <c r="T4" s="18" t="str">
+        <v>grimperium_original_H298_pm7_kJmol</v>
+      </c>
+      <c r="U4" s="18" t="str">
+        <v>grimperium_original_H298_predicted_kcalmol</v>
+      </c>
+      <c r="V4" s="18" t="str">
+        <v>observacao</v>
+      </c>
+      <c r="W4" s="24"/>
+      <c r="X4" s="24"/>
+      <c r="Y4" s="24"/>
+      <c r="Z4" s="24"/>
+      <c r="AA4" s="24"/>
+      <c r="AB4" s="24"/>
+      <c r="AC4" s="24"/>
+      <c r="AD4" s="24"/>
+      <c r="AE4" s="24"/>
+      <c r="AF4" s="24"/>
+      <c r="AG4" s="24"/>
+      <c r="AH4" s="24"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>cbt_001</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Acetic acid</v>
+      </c>
+      <c r="C5" t="str">
+        <v>CC(=O)O</v>
+      </c>
+      <c r="D5" t="str">
+        <v> C2H4O2</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Acids</v>
+      </c>
+      <c r="F5" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" t="str">
+        <v>CRC</v>
+      </c>
+      <c r="H5" s="26" t="n">
+        <v>-432.2</v>
+      </c>
+      <c r="I5" s="26" t="n">
+        <v>-434.88</v>
+      </c>
+      <c r="J5" s="26" t="n">
+        <v>-431.35400000000004</v>
+      </c>
+      <c r="K5" s="26" t="n">
+        <v>-426.861</v>
+      </c>
+      <c r="L5" s="26" t="n">
+        <v>-431.19347</v>
+      </c>
+      <c r="M5" s="26" t="n">
+        <v>-426.94471</v>
+      </c>
+      <c r="N5" s="26" t="n">
+        <v>-427.79466</v>
+      </c>
+      <c r="O5" s="26" t="n">
+        <v>-424.18656</v>
+      </c>
+      <c r="P5" s="26" t="n">
+        <v>4.405339999999967</v>
+      </c>
+      <c r="Q5" s="26" t="str"/>
+      <c r="R5" s="26" t="str"/>
+      <c r="S5" s="26"/>
+      <c r="T5" s="26"/>
+      <c r="U5" s="26"/>
+      <c r="V5" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>cbt_002</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Propanoic acid</v>
+      </c>
+      <c r="C6" t="str">
+        <v>CCC(=O)O</v>
+      </c>
+      <c r="D6" t="str">
+        <v>C3H6O2</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Acids</v>
+      </c>
+      <c r="F6" t="n">
+        <v>11</v>
+      </c>
+      <c r="G6" t="str">
+        <v>CRC</v>
+      </c>
+      <c r="H6" s="26" t="n">
+        <v>-455.7</v>
+      </c>
+      <c r="I6" s="26" t="n">
+        <v>-455.52000000000004</v>
+      </c>
+      <c r="J6" s="26" t="n">
+        <v>-452.117</v>
+      </c>
+      <c r="K6" s="26" t="n">
+        <v>-447.69</v>
+      </c>
+      <c r="L6" s="26" t="n">
+        <v>-456.69109</v>
+      </c>
+      <c r="M6" s="26" t="n">
+        <v>-445.3205</v>
+      </c>
+      <c r="N6" s="26" t="n">
+        <v>-446.53103</v>
+      </c>
+      <c r="O6" s="26" t="n">
+        <v>-443.89516</v>
+      </c>
+      <c r="P6" s="26" t="n">
+        <v>9.168970000000002</v>
+      </c>
+      <c r="Q6" s="26" t="str">
+        <v>mol_01087</v>
+      </c>
+      <c r="R6" s="26" t="str">
+        <v>OK</v>
+      </c>
+      <c r="S6" s="26" t="n">
+        <v>-106.72</v>
+      </c>
+      <c r="T6" s="26" t="n">
+        <v>-446.51648</v>
+      </c>
+      <c r="U6" s="26" t="n">
+        <v>-106.750645</v>
+      </c>
+      <c r="V6" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>cbt_003</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Butyric acid</v>
+      </c>
+      <c r="C7" t="str">
+        <v>CCCC(=O)O</v>
+      </c>
+      <c r="D7" t="str">
+        <v>C4H8O2</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Acids</v>
+      </c>
+      <c r="F7" t="n">
+        <v>14</v>
+      </c>
+      <c r="G7" t="str">
+        <v>PERRY</v>
+      </c>
+      <c r="H7" s="26" t="n">
+        <v>-475.8</v>
+      </c>
+      <c r="I7" s="26" t="n">
+        <v>-476.16</v>
+      </c>
+      <c r="J7" s="26" t="n">
+        <v>-472.88000000000005</v>
+      </c>
+      <c r="K7" s="26" t="n">
+        <v>-468.519</v>
+      </c>
+      <c r="L7" s="26" t="n">
+        <v>-485.54653</v>
+      </c>
+      <c r="M7" s="26" t="n">
+        <v>-467.96146</v>
+      </c>
+      <c r="N7" s="26" t="n">
+        <v>-468.50627</v>
+      </c>
+      <c r="O7" s="26" t="n">
+        <v>-464.59833</v>
+      </c>
+      <c r="P7" s="26" t="n">
+        <v>7.293730000000039</v>
+      </c>
+      <c r="Q7" s="26" t="str">
+        <v>mol_01110</v>
+      </c>
+      <c r="R7" s="26" t="str">
+        <v>OK</v>
+      </c>
+      <c r="S7" s="26" t="n">
+        <v>-111.98</v>
+      </c>
+      <c r="T7" s="26" t="n">
+        <v>-468.52432000000005</v>
+      </c>
+      <c r="U7" s="26" t="n">
+        <v>-111.161337</v>
+      </c>
+      <c r="V7" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>cbt_004</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Pentanoic acid</v>
+      </c>
+      <c r="C8" t="str">
+        <v>CCCCC(=O)O</v>
+      </c>
+      <c r="D8" t="str">
+        <v>C5H10O2</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Acids</v>
+      </c>
+      <c r="F8" t="n">
+        <v>17</v>
+      </c>
+      <c r="G8" t="str">
+        <v>PERRY</v>
+      </c>
+      <c r="H8" s="26" t="n">
+        <v>-491.3</v>
+      </c>
+      <c r="I8" s="26" t="n">
+        <v>-496.8</v>
+      </c>
+      <c r="J8" s="26" t="n">
+        <v>-493.64300000000003</v>
+      </c>
+      <c r="K8" s="26" t="n">
+        <v>-489.348</v>
+      </c>
+      <c r="L8" s="26" t="n">
+        <v>-514.08942</v>
+      </c>
+      <c r="M8" s="26" t="n">
+        <v>-490.54819</v>
+      </c>
+      <c r="N8" s="26" t="n">
+        <v>-489.3534</v>
+      </c>
+      <c r="O8" s="26" t="n">
+        <v>-487.6902</v>
+      </c>
+      <c r="P8" s="26" t="n">
+        <v>1.9465999999999894</v>
+      </c>
+      <c r="Q8" s="26" t="str">
+        <v>mol_01151</v>
+      </c>
+      <c r="R8" s="26" t="str">
+        <v>OK</v>
+      </c>
+      <c r="S8" s="26" t="n">
+        <v>-116.96</v>
+      </c>
+      <c r="T8" s="26" t="n">
+        <v>-489.36064</v>
+      </c>
+      <c r="U8" s="26" t="n">
+        <v>-115.302902</v>
+      </c>
+      <c r="V8" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>cbt_005</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Hexanoic acid</v>
+      </c>
+      <c r="C9" t="str">
+        <v>CCCCCC(=O)O</v>
+      </c>
+      <c r="D9" t="str">
+        <v>C6H12O2</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Acids</v>
+      </c>
+      <c r="F9" t="n">
+        <v>20</v>
+      </c>
+      <c r="G9" t="str">
+        <v>PERRY</v>
+      </c>
+      <c r="H9" s="26" t="n">
+        <v>-511.9</v>
+      </c>
+      <c r="I9" s="26" t="n">
+        <v>-517.44</v>
+      </c>
+      <c r="J9" s="26" t="n">
+        <v>-514.406</v>
+      </c>
+      <c r="K9" s="26" t="n">
+        <v>-510.177</v>
+      </c>
+      <c r="L9" s="26" t="n">
+        <v>-542.79065</v>
+      </c>
+      <c r="M9" s="26" t="n">
+        <v>-513.24139</v>
+      </c>
+      <c r="N9" s="26" t="n">
+        <v>-510.9457</v>
+      </c>
+      <c r="O9" s="26" t="n">
+        <v>-508.62109</v>
+      </c>
+      <c r="P9" s="26" t="n">
+        <v>0.9542999999999893</v>
+      </c>
+      <c r="Q9" s="26" t="str">
+        <v>mol_01511</v>
+      </c>
+      <c r="R9" s="26" t="str">
+        <v>OK</v>
+      </c>
+      <c r="S9" s="26" t="n">
+        <v>-122.12</v>
+      </c>
+      <c r="T9" s="26" t="n">
+        <v>-510.95008</v>
+      </c>
+      <c r="U9" s="26"/>
+      <c r="V9" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>cbt_006</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Heptanoic acid</v>
+      </c>
+      <c r="C10" t="str">
+        <v>CCCCCCC(=O)O</v>
+      </c>
+      <c r="D10" t="str">
+        <v>C7H14O2</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Acids</v>
+      </c>
+      <c r="F10" t="n">
+        <v>23</v>
+      </c>
+      <c r="G10" t="str">
+        <v>PERRY</v>
+      </c>
+      <c r="H10" s="26" t="n">
+        <v>-536.2</v>
+      </c>
+      <c r="I10" s="26" t="n">
+        <v>-538.08</v>
+      </c>
+      <c r="J10" s="26" t="n">
+        <v>-535.169</v>
+      </c>
+      <c r="K10" s="26" t="n">
+        <v>-531.0060000000001</v>
+      </c>
+      <c r="L10" s="26" t="n">
+        <v>-571.46466</v>
+      </c>
+      <c r="M10" s="26" t="n">
+        <v>-535.93561</v>
+      </c>
+      <c r="N10" s="26" t="n">
+        <v>-532.2823</v>
+      </c>
+      <c r="O10" s="26" t="n">
+        <v>-529.4829</v>
+      </c>
+      <c r="P10" s="26" t="n">
+        <v>3.9177000000000817</v>
+      </c>
+      <c r="Q10" s="26" t="str">
+        <v>mol_01999</v>
+      </c>
+      <c r="R10" s="26" t="str">
+        <v>OK</v>
+      </c>
+      <c r="S10" s="26" t="n">
+        <v>-127.22</v>
+      </c>
+      <c r="T10" s="26" t="n">
+        <v>-532.28848</v>
+      </c>
+      <c r="U10" s="26"/>
+      <c r="V10" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>cbt_007</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Octanoic acid</v>
+      </c>
+      <c r="C11" t="str">
+        <v>CCCCCCCC(=O)O</v>
+      </c>
+      <c r="D11" t="str">
+        <v>C8H16O2</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Acids</v>
+      </c>
+      <c r="F11" t="n">
+        <v>26</v>
+      </c>
+      <c r="G11" t="str">
+        <v>PERRY</v>
+      </c>
+      <c r="H11" s="26" t="n">
+        <v>-556</v>
+      </c>
+      <c r="I11" s="26" t="n">
+        <v>-558.72</v>
+      </c>
+      <c r="J11" s="26" t="n">
+        <v>-555.932</v>
+      </c>
+      <c r="K11" s="26" t="n">
+        <v>-551.835</v>
+      </c>
+      <c r="L11" s="26" t="n">
+        <v>-600.16472</v>
+      </c>
+      <c r="M11" s="26" t="n">
+        <v>-558.65708</v>
+      </c>
+      <c r="N11" s="26" t="n">
+        <v>-553.67659</v>
+      </c>
+      <c r="O11" s="26" t="n">
+        <v>-550.37463</v>
+      </c>
+      <c r="P11" s="26" t="n">
+        <v>2.323409999999967</v>
+      </c>
+      <c r="Q11" s="26" t="str">
+        <v>mol_02526</v>
+      </c>
+      <c r="R11" s="26" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S11" s="26"/>
+      <c r="T11" s="26"/>
+      <c r="U11" s="26"/>
+      <c r="V11" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>cbt_008</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Dodecanoic acid</v>
+      </c>
+      <c r="C12" t="str">
+        <v>CCCCCCCCCCCC(=O)O</v>
+      </c>
+      <c r="D12" t="str">
+        <v>C12H24O2</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Acids</v>
+      </c>
+      <c r="F12" t="n">
+        <v>38</v>
+      </c>
+      <c r="G12" t="str">
+        <v>CRC</v>
+      </c>
+      <c r="H12" s="26" t="n">
+        <v>-642</v>
+      </c>
+      <c r="I12" s="26" t="n">
+        <v>-641.2800000000001</v>
+      </c>
+      <c r="J12" s="26" t="n">
+        <v>-638.984</v>
+      </c>
+      <c r="K12" s="26" t="n">
+        <v>-635.1510000000001</v>
+      </c>
+      <c r="L12" s="26" t="n">
+        <v>-711.97551</v>
+      </c>
+      <c r="M12" s="26" t="n">
+        <v>-647.41071</v>
+      </c>
+      <c r="N12" s="26" t="n">
+        <v>-636.75846</v>
+      </c>
+      <c r="O12" s="26" t="n">
+        <v>-630.763</v>
+      </c>
+      <c r="P12" s="26" t="n">
+        <v>5.241539999999986</v>
+      </c>
+      <c r="Q12" s="26" t="str">
+        <v>mol_19014</v>
+      </c>
+      <c r="R12" s="26" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S12" s="26"/>
+      <c r="T12" s="26"/>
+      <c r="U12" s="26"/>
+      <c r="V12" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>cbt_009</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Tetradecanoic acid</v>
+      </c>
+      <c r="C13" t="str">
+        <v>CCCCCCCCCCCCCC(=O)O</v>
+      </c>
+      <c r="D13" t="str">
+        <v>C14H28O2</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Acids</v>
+      </c>
+      <c r="F13" t="n">
+        <v>44</v>
+      </c>
+      <c r="G13" t="str">
+        <v>CRC</v>
+      </c>
+      <c r="H13" s="26" t="n">
+        <v>-693.7</v>
+      </c>
+      <c r="I13" s="26" t="n">
+        <v>-682.5600000000001</v>
+      </c>
+      <c r="J13" s="26" t="n">
+        <v>-680.51</v>
+      </c>
+      <c r="K13" s="26" t="n">
+        <v>-676.809</v>
+      </c>
+      <c r="L13" s="26" t="n">
+        <v>-766.63135</v>
+      </c>
+      <c r="M13" s="26" t="n">
+        <v>-693.91212</v>
+      </c>
+      <c r="N13" s="26" t="n">
+        <v>-678.95566</v>
+      </c>
+      <c r="O13" s="26" t="n">
+        <v>-669.06647</v>
+      </c>
+      <c r="P13" s="26" t="n">
+        <v>14.74434000000008</v>
+      </c>
+      <c r="Q13" s="26" t="str"/>
+      <c r="R13" s="26" t="str"/>
+      <c r="S13" s="26"/>
+      <c r="T13" s="26"/>
+      <c r="U13" s="26"/>
+      <c r="V13" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>cbt_010</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Hexadecanoic acid</v>
+      </c>
+      <c r="C14" t="str">
+        <v>CCCCCCCCCCCCCCCC(=O)O</v>
+      </c>
+      <c r="D14" t="str">
+        <v>C16H32O2</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Acids</v>
+      </c>
+      <c r="F14" t="n">
+        <v>50</v>
+      </c>
+      <c r="G14" t="str">
+        <v>CRC</v>
+      </c>
+      <c r="H14" s="26" t="n">
+        <v>-737.1</v>
+      </c>
+      <c r="I14" s="26" t="n">
+        <v>-723.8400000000001</v>
+      </c>
+      <c r="J14" s="26" t="n">
+        <v>-722.0360000000001</v>
+      </c>
+      <c r="K14" s="26" t="n">
+        <v>-718.467</v>
+      </c>
+      <c r="L14" s="26" t="n">
+        <v>-823.88158</v>
+      </c>
+      <c r="M14" s="26" t="n">
+        <v>-737.15746</v>
+      </c>
+      <c r="N14" s="26" t="n">
+        <v>-721.25162</v>
+      </c>
+      <c r="O14" s="26" t="n">
+        <v>-711.74763</v>
+      </c>
+      <c r="P14" s="26" t="n">
+        <v>15.84838000000002</v>
+      </c>
+      <c r="Q14" s="26" t="str">
+        <v>mol_19005</v>
+      </c>
+      <c r="R14" s="26" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S14" s="26"/>
+      <c r="T14" s="26"/>
+      <c r="U14" s="26"/>
+      <c r="V14" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>cbt_011</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Methanol</v>
+      </c>
+      <c r="C15" t="str">
+        <v>CO</v>
+      </c>
+      <c r="D15" t="str">
+        <v>CH4O</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Alcohols</v>
+      </c>
+      <c r="F15" t="n">
+        <v>6</v>
+      </c>
+      <c r="G15" t="str">
+        <v>PERRY</v>
+      </c>
+      <c r="H15" s="26" t="n">
+        <v>-200.94</v>
+      </c>
+      <c r="I15" s="26" t="n">
+        <v>-216.2</v>
+      </c>
+      <c r="J15" s="26" t="n">
+        <v>-216.534</v>
+      </c>
+      <c r="K15" s="26" t="n">
+        <v>-215.29</v>
+      </c>
+      <c r="L15" s="26" t="n">
+        <v>-238.71117</v>
+      </c>
+      <c r="M15" s="26" t="n">
+        <v>-217.14298</v>
+      </c>
+      <c r="N15" s="26" t="n">
+        <v>-204.75825</v>
+      </c>
+      <c r="O15" s="26" t="n">
+        <v>-209.73142</v>
+      </c>
+      <c r="P15" s="26" t="n">
+        <v>3.818250000000006</v>
+      </c>
+      <c r="Q15" s="26" t="str">
+        <v>mol_05665</v>
+      </c>
+      <c r="R15" s="26" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S15" s="26"/>
+      <c r="T15" s="26"/>
+      <c r="U15" s="26"/>
+      <c r="V15" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>cbt_012</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Ethanol</v>
+      </c>
+      <c r="C16" t="str">
+        <v>CCO</v>
+      </c>
+      <c r="D16" t="str">
+        <v>C2H6O</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Alcohols</v>
+      </c>
+      <c r="F16" t="n">
+        <v>9</v>
+      </c>
+      <c r="G16" t="str">
+        <v>PERRY</v>
+      </c>
+      <c r="H16" s="26" t="n">
+        <v>-234.95</v>
+      </c>
+      <c r="I16" s="26" t="n">
+        <v>-236.83999999999997</v>
+      </c>
+      <c r="J16" s="26" t="n">
+        <v>-237.297</v>
+      </c>
+      <c r="K16" s="26" t="n">
+        <v>-236.119</v>
+      </c>
+      <c r="L16" s="26" t="n">
+        <v>-268.83202</v>
+      </c>
+      <c r="M16" s="26" t="n">
+        <v>-245.83769</v>
+      </c>
+      <c r="N16" s="26" t="n">
+        <v>-242.07799</v>
+      </c>
+      <c r="O16" s="26" t="n">
+        <v>-241.44176</v>
+      </c>
+      <c r="P16" s="26" t="n">
+        <v>7.127990000000011</v>
+      </c>
+      <c r="Q16" s="26" t="str">
+        <v>mol_05309</v>
+      </c>
+      <c r="R16" s="26" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S16" s="26"/>
+      <c r="T16" s="26"/>
+      <c r="U16" s="26"/>
+      <c r="V16" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>cbt_013</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Glycerol</v>
+      </c>
+      <c r="C17" t="str">
+        <v>C(C(CO)O)O</v>
+      </c>
+      <c r="D17" t="str">
+        <v>C3H8O</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Alcohols</v>
+      </c>
+      <c r="F17" t="n">
+        <v>12</v>
+      </c>
+      <c r="G17" t="str">
+        <v>PERRY</v>
+      </c>
+      <c r="H17" s="26" t="n">
+        <v>-577.9</v>
+      </c>
+      <c r="I17" s="26" t="n">
+        <v>-567.22</v>
+      </c>
+      <c r="J17" s="26" t="n">
+        <v>-582.6099999999999</v>
+      </c>
+      <c r="K17" s="26" t="n">
+        <v>-582.7330000000001</v>
+      </c>
+      <c r="L17" s="26" t="n">
+        <v>-665.40715</v>
+      </c>
+      <c r="M17" s="26" t="n">
+        <v>-589.19924</v>
+      </c>
+      <c r="N17" s="26" t="n">
+        <v>-588.45026</v>
+      </c>
+      <c r="O17" s="26" t="n">
+        <v>-595.40912</v>
+      </c>
+      <c r="P17" s="26" t="n">
+        <v>10.55025999999998</v>
+      </c>
+      <c r="Q17" s="26" t="str"/>
+      <c r="R17" s="26" t="str"/>
+      <c r="S17" s="26"/>
+      <c r="T17" s="26"/>
+      <c r="U17" s="26"/>
+      <c r="V17" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>cbt_014</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Propanol</v>
+      </c>
+      <c r="C18" t="str">
+        <v>CCCO</v>
+      </c>
+      <c r="D18" t="str">
+        <v>C3H8O</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Alcohols</v>
+      </c>
+      <c r="F18" t="n">
+        <v>12</v>
+      </c>
+      <c r="G18" t="str">
+        <v>PERRY</v>
+      </c>
+      <c r="H18" s="26" t="n">
+        <v>-254.6</v>
+      </c>
+      <c r="I18" s="26" t="n">
+        <v>-257.47999999999996</v>
+      </c>
+      <c r="J18" s="26" t="n">
+        <v>-258.06</v>
+      </c>
+      <c r="K18" s="26" t="n">
+        <v>-256.94800000000004</v>
+      </c>
+      <c r="L18" s="26" t="n">
+        <v>-297.83885</v>
+      </c>
+      <c r="M18" s="26" t="n">
+        <v>-268.20436</v>
+      </c>
+      <c r="N18" s="26" t="n">
+        <v>-262.4848</v>
+      </c>
+      <c r="O18" s="26" t="n">
+        <v>-262.4955</v>
+      </c>
+      <c r="P18" s="26" t="n">
+        <v>7.884800000000013</v>
+      </c>
+      <c r="Q18" s="26" t="str">
+        <v>mol_05320</v>
+      </c>
+      <c r="R18" s="26" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S18" s="26"/>
+      <c r="T18" s="26"/>
+      <c r="U18" s="26"/>
+      <c r="V18" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>cbt_015</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Butanol</v>
+      </c>
+      <c r="C19" t="str">
+        <v>CCCCO</v>
+      </c>
+      <c r="D19" t="str">
+        <v>C4H10O</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Alcohols</v>
+      </c>
+      <c r="F19" t="n">
+        <v>15</v>
+      </c>
+      <c r="G19" t="str">
+        <v>PERRY</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>-275.1</v>
+      </c>
+      <c r="I19" s="26" t="n">
+        <v>-278.11999999999995</v>
+      </c>
+      <c r="J19" s="26" t="n">
+        <v>-278.82300000000004</v>
+      </c>
+      <c r="K19" s="26" t="n">
+        <v>-277.77700000000004</v>
+      </c>
+      <c r="L19" s="26" t="n">
+        <v>-326.4243</v>
+      </c>
+      <c r="M19" s="26" t="n">
+        <v>-290.86926</v>
+      </c>
+      <c r="N19" s="26" t="n">
+        <v>-283.15306</v>
+      </c>
+      <c r="O19" s="26" t="n">
+        <v>-283.30645</v>
+      </c>
+      <c r="P19" s="26" t="n">
+        <v>8.05305999999996</v>
+      </c>
+      <c r="Q19" s="26" t="str">
+        <v>mol_05337</v>
+      </c>
+      <c r="R19" s="26" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S19" s="26"/>
+      <c r="T19" s="26"/>
+      <c r="U19" s="26"/>
+      <c r="V19" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>cbt_016</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Pentanol</v>
+      </c>
+      <c r="C20" t="str">
+        <v>CCCCCO</v>
+      </c>
+      <c r="D20" t="str">
+        <v>C5H12O</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Alcohols</v>
+      </c>
+      <c r="F20" t="n">
+        <v>18</v>
+      </c>
+      <c r="G20" t="str">
+        <v>PERRY</v>
+      </c>
+      <c r="H20" s="26" t="n">
+        <v>-295.7</v>
+      </c>
+      <c r="I20" s="26" t="n">
+        <v>-298.75999999999993</v>
+      </c>
+      <c r="J20" s="26" t="n">
+        <v>-299.58600000000007</v>
+      </c>
+      <c r="K20" s="26" t="n">
+        <v>-298.60600000000005</v>
+      </c>
+      <c r="L20" s="26" t="n">
+        <v>-355.12297</v>
+      </c>
+      <c r="M20" s="26" t="n">
+        <v>-313.57749</v>
+      </c>
+      <c r="N20" s="26" t="n">
+        <v>-304.42055</v>
+      </c>
+      <c r="O20" s="26" t="n">
+        <v>-304.22328</v>
+      </c>
+      <c r="P20" s="26" t="n">
+        <v>8.720550000000003</v>
+      </c>
+      <c r="Q20" s="26" t="str">
+        <v>mol_05538</v>
+      </c>
+      <c r="R20" s="26" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S20" s="26"/>
+      <c r="T20" s="26"/>
+      <c r="U20" s="26"/>
+      <c r="V20" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>cbt_017</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Hexanol</v>
+      </c>
+      <c r="C21" t="str">
+        <v>CCCCCCO</v>
+      </c>
+      <c r="D21" t="str">
+        <v>C6H14O</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Alcohols</v>
+      </c>
+      <c r="F21" t="n">
+        <v>21</v>
+      </c>
+      <c r="G21" t="str">
+        <v>PERRY</v>
+      </c>
+      <c r="H21" s="26" t="n">
+        <v>-316.2</v>
+      </c>
+      <c r="I21" s="26" t="n">
+        <v>-319.4</v>
+      </c>
+      <c r="J21" s="26" t="n">
+        <v>-320.349</v>
+      </c>
+      <c r="K21" s="26" t="n">
+        <v>-319.43500000000006</v>
+      </c>
+      <c r="L21" s="26" t="n">
+        <v>-383.81376</v>
+      </c>
+      <c r="M21" s="26" t="n">
+        <v>-336.29314</v>
+      </c>
+      <c r="N21" s="26" t="n">
+        <v>-325.86172</v>
+      </c>
+      <c r="O21" s="26" t="n">
+        <v>-325.10002</v>
+      </c>
+      <c r="P21" s="26" t="n">
+        <v>9.661720000000003</v>
+      </c>
+      <c r="Q21" s="26" t="str">
+        <v>mol_05437</v>
+      </c>
+      <c r="R21" s="26" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S21" s="26"/>
+      <c r="T21" s="26"/>
+      <c r="U21" s="26"/>
+      <c r="V21" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>cbt_018</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Heptanol</v>
+      </c>
+      <c r="C22" t="str">
+        <v>CCCCCCCO</v>
+      </c>
+      <c r="D22" t="str">
+        <v>C7H16O</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Alcohols</v>
+      </c>
+      <c r="F22" t="n">
+        <v>24</v>
+      </c>
+      <c r="G22" t="str">
+        <v>PERRY</v>
+      </c>
+      <c r="H22" s="26" t="n">
+        <v>-336.8</v>
+      </c>
+      <c r="I22" s="26" t="n">
+        <v>-340.04</v>
+      </c>
+      <c r="J22" s="26" t="n">
+        <v>-341.112</v>
+      </c>
+      <c r="K22" s="26" t="n">
+        <v>-340.264</v>
+      </c>
+      <c r="L22" s="26" t="n">
+        <v>-412.51169</v>
+      </c>
+      <c r="M22" s="26" t="n">
+        <v>-359.01738</v>
+      </c>
+      <c r="N22" s="26" t="n">
+        <v>-347.16037</v>
+      </c>
+      <c r="O22" s="26" t="n">
+        <v>-345.98604</v>
+      </c>
+      <c r="P22" s="26" t="n">
+        <v>10.360369999999989</v>
+      </c>
+      <c r="Q22" s="26" t="str">
+        <v>mol_05573</v>
+      </c>
+      <c r="R22" s="26" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S22" s="26"/>
+      <c r="T22" s="26"/>
+      <c r="U22" s="26"/>
+      <c r="V22" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>cbt_019</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Octanol</v>
+      </c>
+      <c r="C23" t="str">
+        <v>CCCCCCCCO</v>
+      </c>
+      <c r="D23" t="str">
+        <v>C8H18O</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Alcohols</v>
+      </c>
+      <c r="F23" t="n">
+        <v>27</v>
+      </c>
+      <c r="G23" t="str">
+        <v>PERRY</v>
+      </c>
+      <c r="H23" s="26" t="n">
+        <v>-357.3</v>
+      </c>
+      <c r="I23" s="26" t="n">
+        <v>-360.68</v>
+      </c>
+      <c r="J23" s="26" t="n">
+        <v>-361.87500000000006</v>
+      </c>
+      <c r="K23" s="26" t="n">
+        <v>-361.093</v>
+      </c>
+      <c r="L23" s="26" t="n">
+        <v>-441.21152</v>
+      </c>
+      <c r="M23" s="26" t="n">
+        <v>-381.74613</v>
+      </c>
+      <c r="N23" s="26" t="n">
+        <v>-368.4913</v>
+      </c>
+      <c r="O23" s="26" t="n">
+        <v>-366.87266</v>
+      </c>
+      <c r="P23" s="26" t="n">
+        <v>11.191300000000012</v>
+      </c>
+      <c r="Q23" s="26" t="str"/>
+      <c r="R23" s="26" t="str"/>
+      <c r="S23" s="26"/>
+      <c r="T23" s="26"/>
+      <c r="U23" s="26"/>
+      <c r="V23" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>cbt_020</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Methyl acetate</v>
+      </c>
+      <c r="C24" t="str">
+        <v>CC(=O)OC</v>
+      </c>
+      <c r="D24" t="str">
+        <v>C3H6O2</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Esters</v>
+      </c>
+      <c r="F24" t="n">
+        <v>11</v>
+      </c>
+      <c r="G24" t="str">
+        <v>PERRY</v>
+      </c>
+      <c r="H24" s="26" t="n">
+        <v>-411.9</v>
+      </c>
+      <c r="I24" s="26" t="n">
+        <v>-422.53000000000003</v>
+      </c>
+      <c r="J24" s="26" t="n">
+        <v>-424.84900000000005</v>
+      </c>
+      <c r="K24" s="26" t="n">
+        <v>-424.38800000000003</v>
+      </c>
+      <c r="L24" s="26" t="n">
+        <v>-403.84293</v>
+      </c>
+      <c r="M24" s="26" t="n">
+        <v>-393.95409</v>
+      </c>
+      <c r="N24" s="26" t="n">
+        <v>-405.05317</v>
+      </c>
+      <c r="O24" s="26" t="n">
+        <v>-394.69533</v>
+      </c>
+      <c r="P24" s="26" t="n">
+        <v>6.8468299999999545</v>
+      </c>
+      <c r="Q24" s="26" t="str"/>
+      <c r="R24" s="26" t="str"/>
+      <c r="S24" s="26"/>
+      <c r="T24" s="26"/>
+      <c r="U24" s="26"/>
+      <c r="V24" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>cbt_021</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Methyl propionate</v>
+      </c>
+      <c r="C25" t="str">
+        <v>CCC(=O)OC</v>
+      </c>
+      <c r="D25" t="str">
+        <v>C4H8O2</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Esters</v>
+      </c>
+      <c r="F25" t="n">
+        <v>14</v>
+      </c>
+      <c r="G25" t="str">
+        <v>PERRY</v>
+      </c>
+      <c r="H25" s="26" t="n">
+        <v>-427.5</v>
+      </c>
+      <c r="I25" s="26" t="n">
+        <v>-443.17</v>
+      </c>
+      <c r="J25" s="26" t="n">
+        <v>-440.317</v>
+      </c>
+      <c r="K25" s="26" t="n">
+        <v>-443.61300000000006</v>
+      </c>
+      <c r="L25" s="26" t="n">
+        <v>-429.22249</v>
+      </c>
+      <c r="M25" s="26" t="n">
+        <v>-412.3485</v>
+      </c>
+      <c r="N25" s="26" t="n">
+        <v>-423.65167</v>
+      </c>
+      <c r="O25" s="26" t="n">
+        <v>-414.26053</v>
+      </c>
+      <c r="P25" s="26" t="n">
+        <v>3.848329999999976</v>
+      </c>
+      <c r="Q25" s="26" t="str">
+        <v>mol_03435</v>
+      </c>
+      <c r="R25" s="26" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S25" s="26"/>
+      <c r="T25" s="26"/>
+      <c r="U25" s="26"/>
+      <c r="V25" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>cbt_022</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Methyl butyrate</v>
+      </c>
+      <c r="C26" t="str">
+        <v>CCCC(=O)OC</v>
+      </c>
+      <c r="D26" t="str">
+        <v>C5H10O2</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Esters</v>
+      </c>
+      <c r="F26" t="n">
+        <v>17</v>
+      </c>
+      <c r="G26" t="str">
+        <v>PERRY</v>
+      </c>
+      <c r="H26" s="26" t="n">
+        <v>-450.7</v>
+      </c>
+      <c r="I26" s="26" t="n">
+        <v>-463.81</v>
+      </c>
+      <c r="J26" s="26" t="n">
+        <v>-461.08</v>
+      </c>
+      <c r="K26" s="26" t="n">
+        <v>-464.442</v>
+      </c>
+      <c r="L26" s="26" t="n">
+        <v>-458.04864</v>
+      </c>
+      <c r="M26" s="26" t="n">
+        <v>-434.98867</v>
+      </c>
+      <c r="N26" s="26" t="n">
+        <v>-445.40576</v>
+      </c>
+      <c r="O26" s="26" t="n">
+        <v>-435.46894</v>
+      </c>
+      <c r="P26" s="26" t="n">
+        <v>5.294240000000002</v>
+      </c>
+      <c r="Q26" s="26" t="str">
+        <v>mol_03513</v>
+      </c>
+      <c r="R26" s="26" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S26" s="26"/>
+      <c r="T26" s="26"/>
+      <c r="U26" s="26"/>
+      <c r="V26" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>cbt_023</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Methyl pentanoate</v>
+      </c>
+      <c r="C27" t="str">
+        <v>CCCCC(=O)OC</v>
+      </c>
+      <c r="D27" t="str">
+        <v>C6H12O2</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Esters</v>
+      </c>
+      <c r="F27" t="n">
+        <v>20</v>
+      </c>
+      <c r="G27" t="str">
+        <v>CRC</v>
+      </c>
+      <c r="H27" s="26" t="n">
+        <v>-471.1</v>
+      </c>
+      <c r="I27" s="26" t="n">
+        <v>-484.45</v>
+      </c>
+      <c r="J27" s="26" t="n">
+        <v>-481.843</v>
+      </c>
+      <c r="K27" s="26" t="n">
+        <v>-485.271</v>
+      </c>
+      <c r="L27" s="26" t="n">
+        <v>-486.59503</v>
+      </c>
+      <c r="M27" s="26" t="n">
+        <v>-457.58244</v>
+      </c>
+      <c r="N27" s="26" t="n">
+        <v>-466.21327</v>
+      </c>
+      <c r="O27" s="26" t="n">
+        <v>-455.88914</v>
+      </c>
+      <c r="P27" s="26" t="n">
+        <v>4.88673</v>
+      </c>
+      <c r="Q27" s="26" t="str">
+        <v>mol_03606</v>
+      </c>
+      <c r="R27" s="26" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S27" s="26"/>
+      <c r="T27" s="26"/>
+      <c r="U27" s="26"/>
+      <c r="V27" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>cbt_024</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Methyl hexanoate</v>
+      </c>
+      <c r="C28" t="str">
+        <v>CCCCCC(=O)OC</v>
+      </c>
+      <c r="D28" t="str">
+        <v>C7H14O2</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Esters</v>
+      </c>
+      <c r="F28" t="n">
+        <v>23</v>
+      </c>
+      <c r="G28" t="str">
+        <v>CRC</v>
+      </c>
+      <c r="H28" s="26" t="n">
+        <v>-492.2</v>
+      </c>
+      <c r="I28" s="26" t="n">
+        <v>-505.09</v>
+      </c>
+      <c r="J28" s="26" t="n">
+        <v>-502.60600000000005</v>
+      </c>
+      <c r="K28" s="26" t="n">
+        <v>-506.1</v>
+      </c>
+      <c r="L28" s="26" t="n">
+        <v>-515.29703</v>
+      </c>
+      <c r="M28" s="26" t="n">
+        <v>-480.27905</v>
+      </c>
+      <c r="N28" s="26" t="n">
+        <v>-487.81117</v>
+      </c>
+      <c r="O28" s="26" t="n">
+        <v>-477.20211</v>
+      </c>
+      <c r="P28" s="26" t="n">
+        <v>4.3888299999999845</v>
+      </c>
+      <c r="Q28" s="26" t="str">
+        <v>mol_04136</v>
+      </c>
+      <c r="R28" s="26" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S28" s="26"/>
+      <c r="T28" s="26"/>
+      <c r="U28" s="26"/>
+      <c r="V28" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>cbt_025</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Methyl heptanoate</v>
+      </c>
+      <c r="C29" t="str">
+        <v>CCCCCCC(=O)OC</v>
+      </c>
+      <c r="D29" t="str">
+        <v>C8H16O2</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Esters</v>
+      </c>
+      <c r="F29" t="n">
+        <v>26</v>
+      </c>
+      <c r="G29" t="str">
+        <v>CRC</v>
+      </c>
+      <c r="H29" s="26" t="n">
+        <v>-515.5</v>
+      </c>
+      <c r="I29" s="26" t="n">
+        <v>-525.73</v>
+      </c>
+      <c r="J29" s="26" t="n">
+        <v>-523.3689999999999</v>
+      </c>
+      <c r="K29" s="26" t="n">
+        <v>-526.9290000000001</v>
+      </c>
+      <c r="L29" s="26" t="n">
+        <v>-543.97305</v>
+      </c>
+      <c r="M29" s="26" t="n">
+        <v>-502.97559</v>
+      </c>
+      <c r="N29" s="26" t="n">
+        <v>-509.13106</v>
+      </c>
+      <c r="O29" s="26" t="n">
+        <v>-498.07198</v>
+      </c>
+      <c r="P29" s="26" t="n">
+        <v>6.368940000000009</v>
+      </c>
+      <c r="Q29" s="26" t="str">
+        <v>mol_04742</v>
+      </c>
+      <c r="R29" s="26" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S29" s="26"/>
+      <c r="T29" s="26"/>
+      <c r="U29" s="26"/>
+      <c r="V29" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>cbt_026</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Methyl octanoate</v>
+      </c>
+      <c r="C30" t="str">
+        <v>CCCCCCCC(=O)OC</v>
+      </c>
+      <c r="D30" t="str">
+        <v>C9H18O2</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Esters</v>
+      </c>
+      <c r="F30" t="n">
+        <v>29</v>
+      </c>
+      <c r="G30" t="str">
+        <v>CRC</v>
+      </c>
+      <c r="H30" s="26" t="n">
+        <v>-533.9</v>
+      </c>
+      <c r="I30" s="26" t="n">
+        <v>-546.3700000000001</v>
+      </c>
+      <c r="J30" s="26" t="n">
+        <v>-544.132</v>
+      </c>
+      <c r="K30" s="26" t="n">
+        <v>-547.758</v>
+      </c>
+      <c r="L30" s="26" t="n">
+        <v>-572.67115</v>
+      </c>
+      <c r="M30" s="26" t="n">
+        <v>-525.69852</v>
+      </c>
+      <c r="N30" s="26" t="n">
+        <v>-530.5573</v>
+      </c>
+      <c r="O30" s="26" t="n">
+        <v>-518.94753</v>
+      </c>
+      <c r="P30" s="26" t="n">
+        <v>3.3426999999999225</v>
+      </c>
+      <c r="Q30" s="26" t="str"/>
+      <c r="R30" s="26" t="str"/>
+      <c r="S30" s="26"/>
+      <c r="T30" s="26"/>
+      <c r="U30" s="26"/>
+      <c r="V30" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>cbt_027</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Methyl Dodecanoate</v>
+      </c>
+      <c r="C31" t="str">
+        <v>CCCCCCCCCCCC(=O)OC</v>
+      </c>
+      <c r="D31" t="str">
+        <v>C13H26O2</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Esters</v>
+      </c>
+      <c r="F31" t="n">
+        <v>41</v>
+      </c>
+      <c r="G31" t="str">
+        <v>CRC</v>
+      </c>
+      <c r="H31" s="26" t="n">
+        <v>-617.9</v>
+      </c>
+      <c r="I31" s="26" t="n">
+        <v>-628.9300000000001</v>
+      </c>
+      <c r="J31" s="26" t="n">
+        <v>-627.184</v>
+      </c>
+      <c r="K31" s="26" t="n">
+        <v>-631.0740000000001</v>
+      </c>
+      <c r="L31" s="26" t="n">
+        <v>-687.47505</v>
+      </c>
+      <c r="M31" s="26" t="n">
+        <v>-616.61431</v>
+      </c>
+      <c r="N31" s="26" t="n">
+        <v>-615.92062</v>
+      </c>
+      <c r="O31" s="26" t="n">
+        <v>-602.49831</v>
+      </c>
+      <c r="P31" s="26" t="n">
+        <v>1.979379999999992</v>
+      </c>
+      <c r="Q31" s="26" t="str">
+        <v>mol_19010</v>
+      </c>
+      <c r="R31" s="26" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S31" s="26"/>
+      <c r="T31" s="26"/>
+      <c r="U31" s="26"/>
+      <c r="V31" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>cbt_028</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Methyl Tetradecanoate</v>
+      </c>
+      <c r="C32" t="str">
+        <v>CCCCCCCCCCCCCC(=O)OC</v>
+      </c>
+      <c r="D32" t="str">
+        <v>C15H30O2</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Esters</v>
+      </c>
+      <c r="F32" t="n">
+        <v>47</v>
+      </c>
+      <c r="G32" t="str">
+        <v>CRC</v>
+      </c>
+      <c r="H32" s="26" t="n">
+        <v>-656.9</v>
+      </c>
+      <c r="I32" s="26" t="n">
+        <v>-670.21</v>
+      </c>
+      <c r="J32" s="26" t="n">
+        <v>-668.71</v>
+      </c>
+      <c r="K32" s="26" t="n">
+        <v>-672.732</v>
+      </c>
+      <c r="L32" s="26" t="n">
+        <v>-739.06414</v>
+      </c>
+      <c r="M32" s="26" t="n">
+        <v>-658.6227</v>
+      </c>
+      <c r="N32" s="26" t="n">
+        <v>-656.87245</v>
+      </c>
+      <c r="O32" s="26" t="n">
+        <v>-640.24608</v>
+      </c>
+      <c r="P32" s="26" t="n">
+        <v>0.02755000000001928</v>
+      </c>
+      <c r="Q32" s="26" t="str"/>
+      <c r="R32" s="26" t="str"/>
+      <c r="S32" s="26"/>
+      <c r="T32" s="26"/>
+      <c r="U32" s="26"/>
+      <c r="V32" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>cbt_029</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Methyl Hexadecanoate</v>
+      </c>
+      <c r="C33" t="str">
+        <v>CCCCCCCCCCCCCCCC(=O)OC</v>
+      </c>
+      <c r="D33" t="str">
+        <v>C17H34O2</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Esters</v>
+      </c>
+      <c r="F33" t="n">
+        <v>50</v>
+      </c>
+      <c r="G33" t="str">
+        <v>NIST</v>
+      </c>
+      <c r="H33" s="26" t="n">
+        <v>-665.6</v>
+      </c>
+      <c r="I33" s="26" t="n">
+        <v>-711.49</v>
+      </c>
+      <c r="J33" s="26" t="n">
+        <v>-710.236</v>
+      </c>
+      <c r="K33" s="26" t="n">
+        <v>-714.3900000000001</v>
+      </c>
+      <c r="L33" s="26" t="n">
+        <v>-796.26075</v>
+      </c>
+      <c r="M33" s="26" t="n">
+        <v>-706.07494</v>
+      </c>
+      <c r="N33" s="26" t="n">
+        <v>-698.10851</v>
+      </c>
+      <c r="O33" s="26" t="n">
+        <v>-679.09472</v>
+      </c>
+      <c r="P33" s="26" t="n">
+        <v>32.50851</v>
+      </c>
+      <c r="Q33" s="26" t="str"/>
+      <c r="R33" s="26" t="str"/>
+      <c r="S33" s="26"/>
+      <c r="T33" s="26"/>
+      <c r="U33" s="26"/>
+      <c r="V33" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>cbt_030</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Triacetin</v>
+      </c>
+      <c r="C34" t="str">
+        <v>CC(=O)OCC(COC(C)=O)OC(C)=O</v>
+      </c>
+      <c r="D34" t="str">
+        <v>C9H14O6</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Triglycerides</v>
+      </c>
+      <c r="F34" t="n">
+        <v>29</v>
+      </c>
+      <c r="G34" t="str">
+        <v>CRC</v>
+      </c>
+      <c r="H34" s="26" t="n">
+        <v>-1245</v>
+      </c>
+      <c r="I34" s="26" t="n">
+        <v>-1186.21</v>
+      </c>
+      <c r="J34" s="26" t="n">
+        <v>-1193.078</v>
+      </c>
+      <c r="K34" s="26" t="n">
+        <v>-1202.397</v>
+      </c>
+      <c r="L34" s="26" t="n">
+        <v>-1142.86094</v>
+      </c>
+      <c r="M34" s="26" t="n">
+        <v>-1100.06525</v>
+      </c>
+      <c r="N34" s="26" t="n">
+        <v>-1190.81269</v>
+      </c>
+      <c r="O34" s="26" t="n">
+        <v>-1130.8903</v>
+      </c>
+      <c r="P34" s="26" t="n">
+        <v>54.187310000000025</v>
+      </c>
+      <c r="Q34" s="26" t="str">
+        <v>mol_19015</v>
+      </c>
+      <c r="R34" s="26" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S34" s="26"/>
+      <c r="T34" s="26"/>
+      <c r="U34" s="26"/>
+      <c r="V34" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>cbt_031</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Tributyrin</v>
+      </c>
+      <c r="C35" t="str">
+        <v>CCCC(=O)OCC(COC(=O)CCC)OC(=O)CCC</v>
+      </c>
+      <c r="D35" t="str">
+        <v>C15H26O6</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Triglycerides</v>
+      </c>
+      <c r="F35" t="n">
+        <v>47</v>
+      </c>
+      <c r="G35" t="str">
+        <v>NIST</v>
+      </c>
+      <c r="H35" s="26" t="n">
+        <v>-1388.9</v>
+      </c>
+      <c r="I35" s="26" t="n">
+        <v>-1310.0500000000002</v>
+      </c>
+      <c r="J35" s="26" t="n">
+        <v>-1312.3609999999999</v>
+      </c>
+      <c r="K35" s="26" t="n">
+        <v>-1325.767</v>
+      </c>
+      <c r="L35" s="26" t="n">
+        <v>-1299.98751</v>
+      </c>
+      <c r="M35" s="26" t="n">
+        <v>-1229.83066</v>
+      </c>
+      <c r="N35" s="26" t="n">
+        <v>-1303.39424</v>
+      </c>
+      <c r="O35" s="26" t="n">
+        <v>-1252.52058</v>
+      </c>
+      <c r="P35" s="26" t="n">
+        <v>85.50576000000001</v>
+      </c>
+      <c r="Q35" s="26" t="str"/>
+      <c r="R35" s="26" t="str"/>
+      <c r="S35" s="26"/>
+      <c r="T35" s="26"/>
+      <c r="U35" s="26"/>
+      <c r="V35" t="str">
+        <v>SMILES manual; revisar/canonicalizar com RDKit no grimperium_mini.</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>cbt_036</v>
+      </c>
+      <c r="B40" t="str">
+        <v>9-Octadecenoic acid</v>
+      </c>
+      <c r="C40" t="str">
+        <v>CCCCCCCCC=CCCCCCCCC(=O)O</v>
+      </c>
+      <c r="D40" t="str">
+        <v>C18H34O2</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Acids</v>
+      </c>
+      <c r="F40" t="n">
+        <v>54</v>
+      </c>
+      <c r="H40">
+        <v>-694.4</v>
+      </c>
+      <c r="V40" t="str">
+        <v>Added for grimperium_mini pipeline.</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>cbt_037</v>
+      </c>
+      <c r="B41" t="str">
+        <v>9,12-Octadecadienoic acid</v>
+      </c>
+      <c r="C41" t="str">
+        <v>CCCCCC=CCC=CCCCCCCCC(=O)O</v>
+      </c>
+      <c r="D41" t="str">
+        <v>C18H32O2</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Acids</v>
+      </c>
+      <c r="F41" t="n">
+        <v>52</v>
+      </c>
+      <c r="H41">
+        <v>-561.9</v>
+      </c>
+      <c r="V41" t="str">
+        <v>Added for grimperium_mini pipeline.</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>cbt_038</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Methyl oleate</v>
+      </c>
+      <c r="C42" t="str">
+        <v>CCCCCCCCC=CCCCCCCCC(=O)OC</v>
+      </c>
+      <c r="D42" t="str">
+        <v>C19H36O2</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Esters</v>
+      </c>
+      <c r="F42" t="n">
+        <v>57</v>
+      </c>
+      <c r="H42">
+        <v>-627.1</v>
+      </c>
+      <c r="V42" t="str">
+        <v>Added for grimperium_mini pipeline.</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>cbt_039</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Methyl linoleate</v>
+      </c>
+      <c r="C43" t="str">
+        <v>CCCCCC=CCC=CCCCCCCCC(=O)OC</v>
+      </c>
+      <c r="D43" t="str">
+        <v>C19H34O2</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Esters</v>
+      </c>
+      <c r="F43" t="n">
+        <v>55</v>
+      </c>
+      <c r="H43">
+        <v>-518.8</v>
+      </c>
+      <c r="V43" t="str">
+        <v>Added for grimperium_mini pipeline.</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A1:Y1"/>
+    <mergeCell ref="A2:Y2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>